<commit_message>
Update 김청축_2026_출석부.xlsx via Dashboard
</commit_message>
<xml_diff>
--- a/김청축_2026_출석부.xlsx
+++ b/김청축_2026_출석부.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bcabf36b0134af82/바탕 화면/김인혁_청년축구단/1. 출석부/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1467" documentId="13_ncr:1_{DC8612FD-A52F-4EAD-BD68-700165C8B081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42309875-AC3A-4BC5-83EE-6C35178E488A}"/>
+  <xr:revisionPtr revIDLastSave="1563" documentId="13_ncr:1_{DC8612FD-A52F-4EAD-BD68-700165C8B081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6598F0C0-BF3E-4CB0-8714-D330CE37F57A}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="606" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="606" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="종합Sheet" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3102" uniqueCount="462">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3172" uniqueCount="462">
   <si>
     <t>C/S DF (0.2)</t>
   </si>
@@ -2530,10 +2530,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2542,20 +2542,20 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3508,7 +3508,7 @@
       </c>
       <c r="AS2" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="AT2" s="1">
         <f t="shared" si="1"/>
@@ -3700,7 +3700,9 @@
       <c r="AR3" s="4">
         <v>46303</v>
       </c>
-      <c r="AS3" s="4"/>
+      <c r="AS3" s="4">
+        <v>46310</v>
+      </c>
       <c r="AT3" s="4"/>
       <c r="AU3" s="4"/>
       <c r="AV3" s="4"/>
@@ -3762,11 +3764,11 @@
       </c>
       <c r="H4" s="6">
         <f>I4+개인기록Sheet!C4</f>
-        <v>27.2</v>
+        <v>28.6</v>
       </c>
       <c r="I4" s="6">
         <f>(COUNTIF(J4:CD4,"출전")*1)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>348</v>
@@ -3853,7 +3855,9 @@
       <c r="AR4" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="AS4" s="2"/>
+      <c r="AS4" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT4" s="2"/>
       <c r="AU4" s="2"/>
       <c r="AV4" s="2"/>
@@ -3911,7 +3915,7 @@
       </c>
       <c r="G5" s="2">
         <f t="shared" ref="G5:G35" si="2">RANK(H5,$H$4:$H$122,0)</f>
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H5" s="6">
         <f>I5+개인기록Sheet!C5</f>
@@ -4336,7 +4340,7 @@
       </c>
       <c r="G9" s="2">
         <f t="shared" si="2"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H9" s="6">
         <f>I9+개인기록Sheet!C9</f>
@@ -4455,7 +4459,7 @@
       </c>
       <c r="G10" s="2">
         <f t="shared" si="2"/>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H10" s="6">
         <f>I10+개인기록Sheet!C10</f>
@@ -4592,7 +4596,7 @@
       </c>
       <c r="G11" s="2">
         <f t="shared" si="2"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H11" s="6">
         <f>I11+개인기록Sheet!C11</f>
@@ -5042,7 +5046,7 @@
       </c>
       <c r="G15" s="2">
         <f t="shared" si="2"/>
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H15" s="6">
         <f>I15+개인기록Sheet!C15</f>
@@ -5153,7 +5157,7 @@
       </c>
       <c r="G16" s="2">
         <f t="shared" si="2"/>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H16" s="6">
         <f>I16+개인기록Sheet!C16</f>
@@ -5276,7 +5280,7 @@
       </c>
       <c r="G17" s="2">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H17" s="6">
         <f>I17+개인기록Sheet!C17</f>
@@ -5618,7 +5622,7 @@
       </c>
       <c r="G20" s="2">
         <f t="shared" si="2"/>
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H20" s="6">
         <f>I20+개인기록Sheet!C20</f>
@@ -6044,15 +6048,15 @@
       </c>
       <c r="G24" s="2">
         <f t="shared" si="2"/>
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H24" s="6">
         <f>I24+개인기록Sheet!C24</f>
-        <v>8.1</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="I24" s="6">
         <f t="shared" si="3"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
@@ -6103,7 +6107,9 @@
       <c r="AP24" s="2"/>
       <c r="AQ24" s="2"/>
       <c r="AR24" s="2"/>
-      <c r="AS24" s="2"/>
+      <c r="AS24" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT24" s="2"/>
       <c r="AU24" s="2"/>
       <c r="AV24" s="2"/>
@@ -6161,15 +6167,15 @@
       </c>
       <c r="G25" s="2">
         <f t="shared" si="2"/>
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H25" s="6">
         <f>I25+개인기록Sheet!C25</f>
-        <v>14.9</v>
+        <v>15.9</v>
       </c>
       <c r="I25" s="6">
         <f t="shared" si="3"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J25" s="2"/>
       <c r="K25" s="2" t="s">
@@ -6230,7 +6236,9 @@
       </c>
       <c r="AQ25" s="2"/>
       <c r="AR25" s="2"/>
-      <c r="AS25" s="2"/>
+      <c r="AS25" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT25" s="2"/>
       <c r="AU25" s="2"/>
       <c r="AV25" s="2"/>
@@ -6672,7 +6680,7 @@
       </c>
       <c r="G29" s="2">
         <f t="shared" si="2"/>
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H29" s="6">
         <f>I29+개인기록Sheet!C29</f>
@@ -6781,15 +6789,15 @@
       </c>
       <c r="G30" s="2">
         <f t="shared" si="2"/>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H30" s="6">
         <f>I30+개인기록Sheet!C30</f>
-        <v>18.600000000000001</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="I30" s="6">
         <f t="shared" si="3"/>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J30" s="2"/>
       <c r="K30" s="2" t="s">
@@ -6854,7 +6862,9 @@
       </c>
       <c r="AQ30" s="2"/>
       <c r="AR30" s="2"/>
-      <c r="AS30" s="2"/>
+      <c r="AS30" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT30" s="2"/>
       <c r="AU30" s="2"/>
       <c r="AV30" s="2"/>
@@ -6916,11 +6926,11 @@
       </c>
       <c r="H31" s="6">
         <f>I31+개인기록Sheet!C31</f>
-        <v>31.6</v>
+        <v>32.6</v>
       </c>
       <c r="I31" s="6">
         <f t="shared" si="3"/>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>348</v>
@@ -7009,7 +7019,9 @@
       <c r="AR31" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="AS31" s="2"/>
+      <c r="AS31" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT31" s="2"/>
       <c r="AU31" s="2"/>
       <c r="AV31" s="2"/>
@@ -7067,15 +7079,15 @@
       </c>
       <c r="G32" s="2">
         <f t="shared" si="2"/>
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H32" s="6">
         <f>I32+개인기록Sheet!C32</f>
-        <v>10.4</v>
+        <v>11.4</v>
       </c>
       <c r="I32" s="6">
         <f t="shared" si="3"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J32" s="2"/>
       <c r="K32" s="2" t="s">
@@ -7132,7 +7144,9 @@
         <v>348</v>
       </c>
       <c r="AR32" s="2"/>
-      <c r="AS32" s="2"/>
+      <c r="AS32" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT32" s="2"/>
       <c r="AU32" s="2"/>
       <c r="AV32" s="2"/>
@@ -7190,7 +7204,7 @@
       </c>
       <c r="G33" s="2">
         <f t="shared" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H33" s="6">
         <f>I33+개인기록Sheet!C33</f>
@@ -7435,7 +7449,7 @@
       </c>
       <c r="G35" s="2">
         <f t="shared" si="2"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H35" s="6">
         <f>I35+개인기록Sheet!C35</f>
@@ -7578,7 +7592,7 @@
       </c>
       <c r="G36" s="2">
         <f t="shared" ref="G36:G67" si="6">RANK(H36,$H$4:$H$122,0)</f>
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H36" s="6">
         <f>I36+개인기록Sheet!C36</f>
@@ -7801,7 +7815,7 @@
       </c>
       <c r="G38" s="2">
         <f t="shared" si="6"/>
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H38" s="6">
         <f>I38+개인기록Sheet!C38</f>
@@ -8116,7 +8130,7 @@
       </c>
       <c r="G41" s="2">
         <f t="shared" si="6"/>
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H41" s="6">
         <f>I41+개인기록Sheet!C41</f>
@@ -8223,15 +8237,15 @@
       </c>
       <c r="G42" s="2">
         <f t="shared" si="6"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H42" s="6">
         <f>I42+개인기록Sheet!C42</f>
-        <v>26.6</v>
+        <v>27.8</v>
       </c>
       <c r="I42" s="6">
         <f t="shared" si="3"/>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J42" s="2"/>
       <c r="K42" s="2" t="s">
@@ -8312,7 +8326,9 @@
       <c r="AR42" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="AS42" s="2"/>
+      <c r="AS42" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT42" s="2"/>
       <c r="AU42" s="2"/>
       <c r="AV42" s="2"/>
@@ -8370,7 +8386,7 @@
       </c>
       <c r="G43" s="2">
         <f t="shared" si="6"/>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H43" s="6">
         <f>I43+개인기록Sheet!C43</f>
@@ -8493,15 +8509,15 @@
       </c>
       <c r="G44" s="2">
         <f t="shared" si="6"/>
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="H44" s="6">
         <f>I44+개인기록Sheet!C44</f>
-        <v>8.4</v>
+        <v>10.600000000000001</v>
       </c>
       <c r="I44" s="6">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
@@ -8550,7 +8566,9 @@
       </c>
       <c r="AQ44" s="2"/>
       <c r="AR44" s="2"/>
-      <c r="AS44" s="2"/>
+      <c r="AS44" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT44" s="2"/>
       <c r="AU44" s="2"/>
       <c r="AV44" s="2"/>
@@ -8710,15 +8728,15 @@
       </c>
       <c r="G46" s="2">
         <f t="shared" si="6"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H46" s="6">
         <f>I46+개인기록Sheet!C46</f>
-        <v>21.4</v>
+        <v>22.6</v>
       </c>
       <c r="I46" s="6">
         <f t="shared" si="3"/>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J46" s="2"/>
       <c r="K46" s="2" t="s">
@@ -8791,7 +8809,9 @@
         <v>348</v>
       </c>
       <c r="AR46" s="2"/>
-      <c r="AS46" s="2"/>
+      <c r="AS46" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT46" s="2"/>
       <c r="AU46" s="2"/>
       <c r="AV46" s="2"/>
@@ -8842,7 +8862,7 @@
       </c>
       <c r="D47" s="54">
         <f t="shared" ref="D47:D49" si="8">COUNTA(AF47:AU47)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E47" s="54"/>
       <c r="F47" s="2" t="s">
@@ -8850,15 +8870,15 @@
       </c>
       <c r="G47" s="2">
         <f t="shared" si="6"/>
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="H47" s="6">
         <f>I47+개인기록Sheet!C47</f>
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="I47" s="6">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
@@ -8899,7 +8919,9 @@
       <c r="AP47" s="2"/>
       <c r="AQ47" s="2"/>
       <c r="AR47" s="2"/>
-      <c r="AS47" s="2"/>
+      <c r="AS47" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT47" s="2"/>
       <c r="AU47" s="2"/>
       <c r="AV47" s="2"/>
@@ -9165,7 +9187,7 @@
       </c>
       <c r="G50" s="2">
         <f t="shared" si="6"/>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H50" s="6">
         <f>I50+개인기록Sheet!C50</f>
@@ -9403,7 +9425,7 @@
       </c>
       <c r="G52" s="2">
         <f t="shared" si="6"/>
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H52" s="6">
         <f>I52+개인기록Sheet!C52</f>
@@ -9517,7 +9539,7 @@
       </c>
       <c r="G53" s="2">
         <f t="shared" si="6"/>
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H53" s="6">
         <f>I53+개인기록Sheet!C53</f>
@@ -9842,11 +9864,11 @@
       </c>
       <c r="H56" s="6">
         <f>I56+개인기록Sheet!C56</f>
-        <v>24.6</v>
+        <v>25.6</v>
       </c>
       <c r="I56" s="6">
         <f t="shared" si="3"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J56" s="2"/>
       <c r="K56" s="2" t="s">
@@ -9925,7 +9947,9 @@
       <c r="AR56" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="AS56" s="2"/>
+      <c r="AS56" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT56" s="2"/>
       <c r="AU56" s="2"/>
       <c r="AV56" s="2"/>
@@ -9983,15 +10007,15 @@
       </c>
       <c r="G57" s="2">
         <f t="shared" si="6"/>
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="H57" s="6">
         <f>I57+개인기록Sheet!C57</f>
-        <v>3.6</v>
+        <v>5.2</v>
       </c>
       <c r="I57" s="6">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J57" s="2" t="s">
         <v>348</v>
@@ -10034,7 +10058,9 @@
       <c r="AP57" s="2"/>
       <c r="AQ57" s="2"/>
       <c r="AR57" s="2"/>
-      <c r="AS57" s="2"/>
+      <c r="AS57" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT57" s="2"/>
       <c r="AU57" s="2"/>
       <c r="AV57" s="2"/>
@@ -10092,7 +10118,7 @@
       </c>
       <c r="G58" s="2">
         <f t="shared" si="6"/>
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H58" s="6">
         <f>I58+개인기록Sheet!C58</f>
@@ -10317,15 +10343,15 @@
       </c>
       <c r="G60" s="2">
         <f t="shared" si="6"/>
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H60" s="6">
         <f>I60+개인기록Sheet!C60</f>
-        <v>3.6</v>
+        <v>4.8</v>
       </c>
       <c r="I60" s="6">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J60" s="2"/>
       <c r="K60" s="2" t="s">
@@ -10368,7 +10394,9 @@
       <c r="AP60" s="2"/>
       <c r="AQ60" s="2"/>
       <c r="AR60" s="2"/>
-      <c r="AS60" s="2"/>
+      <c r="AS60" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT60" s="2"/>
       <c r="AU60" s="2"/>
       <c r="AV60" s="2"/>
@@ -10671,7 +10699,7 @@
       </c>
       <c r="G63" s="2">
         <f t="shared" si="6"/>
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H63" s="6">
         <f>I63+개인기록Sheet!C63</f>
@@ -11211,7 +11239,7 @@
       </c>
       <c r="G68" s="2">
         <f t="shared" ref="G68:G99" si="12">RANK(H68,$H$4:$H$122,0)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H68" s="6">
         <f>I68+개인기록Sheet!C68</f>
@@ -11347,7 +11375,7 @@
       </c>
       <c r="G69" s="2">
         <f t="shared" si="12"/>
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H69" s="6">
         <f>I69+개인기록Sheet!C69</f>
@@ -11458,15 +11486,15 @@
       </c>
       <c r="G70" s="2">
         <f t="shared" si="12"/>
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H70" s="6">
         <f>I70+개인기록Sheet!C70</f>
-        <v>6.8</v>
+        <v>8</v>
       </c>
       <c r="I70" s="6">
         <f t="shared" si="11"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J70" s="2"/>
       <c r="K70" s="2"/>
@@ -11515,7 +11543,9 @@
       <c r="AP70" s="2"/>
       <c r="AQ70" s="2"/>
       <c r="AR70" s="2"/>
-      <c r="AS70" s="2"/>
+      <c r="AS70" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT70" s="2"/>
       <c r="AU70" s="2"/>
       <c r="AV70" s="2"/>
@@ -11573,7 +11603,7 @@
       </c>
       <c r="G71" s="2">
         <f t="shared" si="12"/>
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H71" s="6">
         <f>I71+개인기록Sheet!C71</f>
@@ -11796,7 +11826,7 @@
       </c>
       <c r="G73" s="2">
         <f t="shared" si="12"/>
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H73" s="6">
         <f>I73+개인기록Sheet!C73</f>
@@ -11909,15 +11939,15 @@
       </c>
       <c r="G74" s="2">
         <f t="shared" si="12"/>
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="H74" s="6">
         <f>I74+개인기록Sheet!C74</f>
-        <v>6.6</v>
+        <v>7.8</v>
       </c>
       <c r="I74" s="6">
         <f t="shared" si="11"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J74" s="2"/>
       <c r="K74" s="2" t="s">
@@ -11964,7 +11994,9 @@
       <c r="AP74" s="2"/>
       <c r="AQ74" s="2"/>
       <c r="AR74" s="2"/>
-      <c r="AS74" s="2"/>
+      <c r="AS74" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT74" s="2"/>
       <c r="AU74" s="2"/>
       <c r="AV74" s="2"/>
@@ -12022,7 +12054,7 @@
       </c>
       <c r="G75" s="2">
         <f t="shared" si="12"/>
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H75" s="6">
         <f>I75+개인기록Sheet!C75</f>
@@ -12246,7 +12278,7 @@
       </c>
       <c r="G77" s="2">
         <f t="shared" si="12"/>
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H77" s="6">
         <f>I77+개인기록Sheet!C77</f>
@@ -12353,7 +12385,7 @@
       </c>
       <c r="G78" s="2">
         <f t="shared" si="12"/>
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H78" s="6">
         <f>I78+개인기록Sheet!C78</f>
@@ -12474,7 +12506,7 @@
       </c>
       <c r="G79" s="2">
         <f t="shared" si="12"/>
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H79" s="6">
         <f>I79+개인기록Sheet!C79</f>
@@ -12589,15 +12621,15 @@
       </c>
       <c r="G80" s="2">
         <f t="shared" si="12"/>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H80" s="6">
         <f>I80+개인기록Sheet!C80</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I80" s="6">
         <f t="shared" si="11"/>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J80" s="2"/>
       <c r="K80" s="2"/>
@@ -12660,7 +12692,9 @@
       </c>
       <c r="AQ80" s="2"/>
       <c r="AR80" s="2"/>
-      <c r="AS80" s="2"/>
+      <c r="AS80" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT80" s="2"/>
       <c r="AU80" s="2"/>
       <c r="AV80" s="2"/>
@@ -12718,15 +12752,15 @@
       </c>
       <c r="G81" s="2">
         <f t="shared" si="12"/>
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="H81" s="6">
         <f>I81+개인기록Sheet!C81</f>
-        <v>14.6</v>
+        <v>16</v>
       </c>
       <c r="I81" s="6">
         <f t="shared" si="11"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J81" s="2"/>
       <c r="K81" s="2"/>
@@ -12787,7 +12821,9 @@
         <v>348</v>
       </c>
       <c r="AR81" s="2"/>
-      <c r="AS81" s="2"/>
+      <c r="AS81" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT81" s="2"/>
       <c r="AU81" s="2"/>
       <c r="AV81" s="2"/>
@@ -12845,7 +12881,7 @@
       </c>
       <c r="G82" s="2">
         <f t="shared" si="12"/>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H82" s="6">
         <f>I82+개인기록Sheet!C82</f>
@@ -12970,15 +13006,15 @@
       </c>
       <c r="G83" s="2">
         <f t="shared" si="12"/>
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H83" s="6">
         <f>I83+개인기록Sheet!C83</f>
-        <v>15</v>
+        <v>16.2</v>
       </c>
       <c r="I83" s="6">
         <f t="shared" si="11"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J83" s="2"/>
       <c r="K83" s="2"/>
@@ -13039,7 +13075,9 @@
       <c r="AR83" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="AS83" s="2"/>
+      <c r="AS83" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT83" s="2"/>
       <c r="AU83" s="2"/>
       <c r="AV83" s="2"/>
@@ -13097,7 +13135,7 @@
       </c>
       <c r="G84" s="2">
         <f t="shared" si="12"/>
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H84" s="6">
         <f>I84+개인기록Sheet!C84</f>
@@ -13208,7 +13246,7 @@
       </c>
       <c r="G85" s="2">
         <f t="shared" si="12"/>
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H85" s="6">
         <f>I85+개인기록Sheet!C85</f>
@@ -13325,7 +13363,7 @@
       </c>
       <c r="G86" s="2">
         <f t="shared" si="12"/>
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H86" s="6">
         <f>I86+개인기록Sheet!C86</f>
@@ -13542,7 +13580,7 @@
       </c>
       <c r="G88" s="2">
         <f t="shared" si="12"/>
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H88" s="6">
         <f>I88+개인기록Sheet!C88</f>
@@ -13651,7 +13689,7 @@
       </c>
       <c r="G89" s="2">
         <f t="shared" si="12"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H89" s="6">
         <f>I89+개인기록Sheet!C89</f>
@@ -13972,7 +14010,7 @@
       </c>
       <c r="G92" s="2">
         <f t="shared" si="12"/>
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H92" s="6">
         <f>I92+개인기록Sheet!C92</f>
@@ -14186,15 +14224,15 @@
       </c>
       <c r="G94" s="2">
         <f t="shared" si="12"/>
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H94" s="6">
         <f>I94+개인기록Sheet!C94</f>
-        <v>15.9</v>
+        <v>17.5</v>
       </c>
       <c r="I94" s="6">
         <f t="shared" si="11"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J94" s="2"/>
       <c r="K94" s="2"/>
@@ -14255,7 +14293,9 @@
         <v>348</v>
       </c>
       <c r="AR94" s="2"/>
-      <c r="AS94" s="2"/>
+      <c r="AS94" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT94" s="2"/>
       <c r="AU94" s="2"/>
       <c r="AV94" s="2"/>
@@ -14313,7 +14353,7 @@
       </c>
       <c r="G95" s="2">
         <f t="shared" si="12"/>
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H95" s="6">
         <f>I95+개인기록Sheet!C95</f>
@@ -14526,7 +14566,7 @@
       </c>
       <c r="G97" s="2">
         <f t="shared" si="12"/>
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H97" s="6">
         <f>I97+개인기록Sheet!C97</f>
@@ -14759,7 +14799,7 @@
       </c>
       <c r="G99" s="2">
         <f t="shared" si="12"/>
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H99" s="6">
         <f>I99+개인기록Sheet!C99</f>
@@ -14872,15 +14912,15 @@
       </c>
       <c r="G100" s="2">
         <f t="shared" ref="G100:G122" si="15">RANK(H100,$H$4:$H$122,0)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H100" s="6">
         <f>I100+개인기록Sheet!C100</f>
-        <v>22.6</v>
+        <v>23.8</v>
       </c>
       <c r="I100" s="6">
         <f t="shared" si="11"/>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J100" s="2"/>
       <c r="K100" s="2"/>
@@ -14951,7 +14991,9 @@
       <c r="AR100" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="AS100" s="2"/>
+      <c r="AS100" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT100" s="2"/>
       <c r="AU100" s="2"/>
       <c r="AV100" s="2"/>
@@ -15009,15 +15051,15 @@
       </c>
       <c r="G101" s="2">
         <f t="shared" si="15"/>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H101" s="6">
         <f>I101+개인기록Sheet!C101</f>
-        <v>20.2</v>
+        <v>21.4</v>
       </c>
       <c r="I101" s="6">
         <f t="shared" si="11"/>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J101" s="2"/>
       <c r="K101" s="2"/>
@@ -15086,7 +15128,9 @@
       <c r="AR101" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="AS101" s="2"/>
+      <c r="AS101" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT101" s="2"/>
       <c r="AU101" s="2"/>
       <c r="AV101" s="2"/>
@@ -15144,15 +15188,15 @@
       </c>
       <c r="G102" s="2">
         <f t="shared" si="15"/>
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H102" s="6">
         <f>I102+개인기록Sheet!C102</f>
-        <v>9.5</v>
+        <v>10.7</v>
       </c>
       <c r="I102" s="6">
         <f t="shared" si="11"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J102" s="2"/>
       <c r="K102" s="2"/>
@@ -15205,7 +15249,9 @@
       <c r="AP102" s="2"/>
       <c r="AQ102" s="2"/>
       <c r="AR102" s="2"/>
-      <c r="AS102" s="2"/>
+      <c r="AS102" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT102" s="2"/>
       <c r="AU102" s="2"/>
       <c r="AV102" s="2"/>
@@ -15267,11 +15313,11 @@
       </c>
       <c r="H103" s="6">
         <f>I103+개인기록Sheet!C103</f>
-        <v>30.7</v>
+        <v>32</v>
       </c>
       <c r="I103" s="6">
         <f t="shared" si="11"/>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J103" s="2" t="s">
         <v>348</v>
@@ -15356,7 +15402,9 @@
       <c r="AR103" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="AS103" s="2"/>
+      <c r="AS103" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT103" s="2"/>
       <c r="AU103" s="2"/>
       <c r="AV103" s="2"/>
@@ -15418,11 +15466,11 @@
       </c>
       <c r="H104" s="6">
         <f>I104+개인기록Sheet!C104</f>
-        <v>22</v>
+        <v>23.2</v>
       </c>
       <c r="I104" s="6">
         <f t="shared" si="11"/>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J104" s="2" t="s">
         <v>348</v>
@@ -15497,7 +15545,9 @@
       <c r="AR104" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="AS104" s="2"/>
+      <c r="AS104" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT104" s="2"/>
       <c r="AU104" s="2"/>
       <c r="AV104" s="2"/>
@@ -15555,7 +15605,7 @@
       </c>
       <c r="G105" s="2">
         <f t="shared" si="15"/>
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H105" s="6">
         <f>I105+개인기록Sheet!C105</f>
@@ -15669,7 +15719,7 @@
       </c>
       <c r="G106" s="2">
         <f t="shared" si="15"/>
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H106" s="6">
         <f>I106+개인기록Sheet!C106</f>
@@ -15776,7 +15826,7 @@
       </c>
       <c r="G107" s="2">
         <f t="shared" si="15"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H107" s="6">
         <f>I107+개인기록Sheet!C107</f>
@@ -16007,7 +16057,7 @@
       </c>
       <c r="G109" s="2">
         <f t="shared" si="15"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H109" s="6">
         <f>I109+개인기록Sheet!C109</f>
@@ -16138,7 +16188,7 @@
       </c>
       <c r="G110" s="2">
         <f t="shared" si="15"/>
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="H110" s="6">
         <f>I110+개인기록Sheet!C110</f>
@@ -16390,7 +16440,7 @@
       </c>
       <c r="G112" s="2">
         <f t="shared" si="15"/>
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H112" s="6">
         <f>I112+개인기록Sheet!C112</f>
@@ -16505,7 +16555,7 @@
       </c>
       <c r="G113" s="2">
         <f t="shared" si="15"/>
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H113" s="6">
         <f>I113+개인기록Sheet!C113</f>
@@ -16620,7 +16670,7 @@
       </c>
       <c r="G114" s="2">
         <f t="shared" si="15"/>
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H114" s="6">
         <f>I114+개인기록Sheet!C114</f>
@@ -16727,7 +16777,7 @@
       </c>
       <c r="G115" s="2">
         <f t="shared" si="15"/>
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H115" s="6">
         <f>I115+개인기록Sheet!C115</f>
@@ -16840,7 +16890,7 @@
       </c>
       <c r="G116" s="2">
         <f t="shared" si="15"/>
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H116" s="6">
         <f>I116+개인기록Sheet!C116</f>
@@ -17073,7 +17123,7 @@
       </c>
       <c r="G118" s="2">
         <f t="shared" si="15"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H118" s="6">
         <f>I118+개인기록Sheet!C118</f>
@@ -17391,15 +17441,15 @@
       </c>
       <c r="G121" s="2">
         <f t="shared" si="15"/>
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H121" s="6">
         <f>I121+개인기록Sheet!C121</f>
-        <v>13.2</v>
+        <v>14.8</v>
       </c>
       <c r="I121" s="6">
         <f t="shared" si="11"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J121" s="2"/>
       <c r="K121" s="2" t="s">
@@ -17454,7 +17504,9 @@
       </c>
       <c r="AQ121" s="2"/>
       <c r="AR121" s="2"/>
-      <c r="AS121" s="2"/>
+      <c r="AS121" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT121" s="2"/>
       <c r="AU121" s="2"/>
       <c r="AV121" s="2"/>
@@ -17505,7 +17557,7 @@
       </c>
       <c r="D122" s="54">
         <f>COUNTA(AF122:AU122)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E122" s="54"/>
       <c r="F122" s="2" t="s">
@@ -17513,15 +17565,15 @@
       </c>
       <c r="G122" s="2">
         <f t="shared" si="15"/>
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="H122" s="6">
         <f>I122+개인기록Sheet!C122</f>
-        <v>4.8</v>
+        <v>6.6</v>
       </c>
       <c r="I122" s="6">
         <f t="shared" si="11"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J122" s="2"/>
       <c r="K122" s="2"/>
@@ -17566,7 +17618,9 @@
       <c r="AR122" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="AS122" s="2"/>
+      <c r="AS122" s="2" t="s">
+        <v>348</v>
+      </c>
       <c r="AT122" s="2"/>
       <c r="AU122" s="2"/>
       <c r="AV122" s="2"/>
@@ -17606,7 +17660,6 @@
       <c r="CD122" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:CT122" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="D4:E122">
     <cfRule type="containsText" dxfId="13" priority="1" operator="containsText" text="지급">
@@ -17630,7 +17683,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A2:V328"/>
+  <dimension ref="A2:V340"/>
   <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="15.6" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.8984375" style="1" bestFit="1" customWidth="1"/>
@@ -27019,99 +27072,699 @@
       <c r="U328" s="2"/>
       <c r="V328" s="2"/>
     </row>
+    <row r="331" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B331" s="11">
+        <v>46310</v>
+      </c>
+      <c r="C331" s="10" t="s">
+        <v>394</v>
+      </c>
+      <c r="D331" s="10" t="s">
+        <v>393</v>
+      </c>
+      <c r="E331" s="77" t="s">
+        <v>82</v>
+      </c>
+      <c r="F331" s="77"/>
+      <c r="G331" s="77"/>
+      <c r="H331" s="77"/>
+      <c r="I331" s="78" t="s">
+        <v>85</v>
+      </c>
+      <c r="J331" s="78"/>
+      <c r="K331" s="78"/>
+      <c r="L331" s="78"/>
+      <c r="M331" s="79" t="s">
+        <v>84</v>
+      </c>
+      <c r="N331" s="79"/>
+      <c r="O331" s="79"/>
+      <c r="P331" s="79"/>
+      <c r="Q331" s="80" t="s">
+        <v>78</v>
+      </c>
+      <c r="R331" s="80"/>
+      <c r="S331" s="80"/>
+      <c r="T331" s="80"/>
+      <c r="U331" s="80"/>
+      <c r="V331" s="80"/>
+    </row>
+    <row r="332" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B332" s="73" t="s">
+        <v>65</v>
+      </c>
+      <c r="C332" s="75">
+        <v>0</v>
+      </c>
+      <c r="D332" s="75">
+        <v>1</v>
+      </c>
+      <c r="E332" s="7"/>
+      <c r="F332" s="7"/>
+      <c r="G332" s="7"/>
+      <c r="H332" s="7"/>
+      <c r="I332" s="8"/>
+      <c r="J332" s="8"/>
+      <c r="K332" s="8"/>
+      <c r="L332" s="8"/>
+      <c r="M332" s="20"/>
+      <c r="N332" s="20"/>
+      <c r="O332" s="20"/>
+      <c r="P332" s="20"/>
+      <c r="Q332" s="9"/>
+      <c r="R332" s="9"/>
+      <c r="S332" s="9"/>
+      <c r="T332" s="9"/>
+      <c r="U332" s="9"/>
+      <c r="V332" s="13"/>
+    </row>
+    <row r="333" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B333" s="74"/>
+      <c r="C333" s="76"/>
+      <c r="D333" s="76"/>
+      <c r="E333" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="F333" s="7"/>
+      <c r="G333" s="7"/>
+      <c r="H333" s="7"/>
+      <c r="I333" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="J333" s="8"/>
+      <c r="K333" s="8"/>
+      <c r="L333" s="8"/>
+      <c r="M333" s="20" t="s">
+        <v>219</v>
+      </c>
+      <c r="N333" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="O333" s="20" t="s">
+        <v>307</v>
+      </c>
+      <c r="P333" s="20"/>
+      <c r="Q333" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="R333" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="S333" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="T333" s="9" t="s">
+        <v>351</v>
+      </c>
+      <c r="U333" s="9"/>
+      <c r="V333" s="13" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="334" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B334" s="73" t="s">
+        <v>71</v>
+      </c>
+      <c r="C334" s="75">
+        <v>0</v>
+      </c>
+      <c r="D334" s="75">
+        <v>0</v>
+      </c>
+      <c r="E334" s="7"/>
+      <c r="F334" s="7"/>
+      <c r="G334" s="7"/>
+      <c r="H334" s="7"/>
+      <c r="I334" s="8"/>
+      <c r="J334" s="8"/>
+      <c r="K334" s="8"/>
+      <c r="L334" s="8"/>
+      <c r="M334" s="20"/>
+      <c r="N334" s="20"/>
+      <c r="O334" s="20"/>
+      <c r="P334" s="20"/>
+      <c r="Q334" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="R334" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="S334" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="T334" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="U334" s="9"/>
+      <c r="V334" s="13" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="335" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B335" s="74"/>
+      <c r="C335" s="76"/>
+      <c r="D335" s="76"/>
+      <c r="E335" s="7"/>
+      <c r="F335" s="7"/>
+      <c r="G335" s="7"/>
+      <c r="H335" s="7"/>
+      <c r="I335" s="8"/>
+      <c r="J335" s="8"/>
+      <c r="K335" s="8"/>
+      <c r="L335" s="8"/>
+      <c r="M335" s="20"/>
+      <c r="N335" s="20"/>
+      <c r="O335" s="20"/>
+      <c r="P335" s="20"/>
+      <c r="Q335" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="R335" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="S335" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="T335" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="U335" s="9"/>
+      <c r="V335" s="13" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="336" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B336" s="73" t="s">
+        <v>73</v>
+      </c>
+      <c r="C336" s="75">
+        <v>2</v>
+      </c>
+      <c r="D336" s="75">
+        <v>1</v>
+      </c>
+      <c r="E336" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="F336" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G336" s="7"/>
+      <c r="H336" s="7"/>
+      <c r="I336" s="8"/>
+      <c r="J336" s="8"/>
+      <c r="K336" s="8"/>
+      <c r="L336" s="8"/>
+      <c r="M336" s="20"/>
+      <c r="N336" s="20"/>
+      <c r="O336" s="20"/>
+      <c r="P336" s="20"/>
+      <c r="Q336" s="9"/>
+      <c r="R336" s="9"/>
+      <c r="S336" s="9"/>
+      <c r="T336" s="9"/>
+      <c r="U336" s="9"/>
+      <c r="V336" s="13"/>
+    </row>
+    <row r="337" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B337" s="74"/>
+      <c r="C337" s="76"/>
+      <c r="D337" s="76"/>
+      <c r="E337" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="F337" s="7"/>
+      <c r="G337" s="7"/>
+      <c r="H337" s="7"/>
+      <c r="I337" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="J337" s="8"/>
+      <c r="K337" s="8"/>
+      <c r="L337" s="8"/>
+      <c r="M337" s="20"/>
+      <c r="N337" s="20"/>
+      <c r="O337" s="20"/>
+      <c r="P337" s="20"/>
+      <c r="Q337" s="9"/>
+      <c r="R337" s="9"/>
+      <c r="S337" s="9"/>
+      <c r="T337" s="9"/>
+      <c r="U337" s="9"/>
+      <c r="V337" s="13"/>
+    </row>
+    <row r="338" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B338" s="73" t="s">
+        <v>41</v>
+      </c>
+      <c r="C338" s="75">
+        <v>1</v>
+      </c>
+      <c r="D338" s="75">
+        <v>4</v>
+      </c>
+      <c r="E338" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="F338" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="G338" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="H338" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="I338" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="J338" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="K338" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="L338" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="M338" s="20" t="s">
+        <v>307</v>
+      </c>
+      <c r="N338" s="20" t="s">
+        <v>219</v>
+      </c>
+      <c r="O338" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="P338" s="20"/>
+      <c r="Q338" s="9"/>
+      <c r="R338" s="9"/>
+      <c r="S338" s="9"/>
+      <c r="T338" s="9"/>
+      <c r="U338" s="9"/>
+      <c r="V338" s="13"/>
+    </row>
+    <row r="339" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B339" s="74"/>
+      <c r="C339" s="76"/>
+      <c r="D339" s="76"/>
+      <c r="E339" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="F339" s="7"/>
+      <c r="G339" s="7"/>
+      <c r="H339" s="7"/>
+      <c r="I339" s="8"/>
+      <c r="J339" s="8"/>
+      <c r="K339" s="8"/>
+      <c r="L339" s="8"/>
+      <c r="M339" s="20"/>
+      <c r="N339" s="20"/>
+      <c r="O339" s="20"/>
+      <c r="P339" s="20"/>
+      <c r="Q339" s="9"/>
+      <c r="R339" s="9"/>
+      <c r="S339" s="9"/>
+      <c r="T339" s="9"/>
+      <c r="U339" s="9"/>
+      <c r="V339" s="13"/>
+    </row>
+    <row r="340" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B340" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C340" s="2">
+        <f>SUM(C332:C339)</f>
+        <v>3</v>
+      </c>
+      <c r="D340" s="2">
+        <f>SUM(D332:D339)</f>
+        <v>6</v>
+      </c>
+      <c r="E340" s="2"/>
+      <c r="F340" s="2"/>
+      <c r="G340" s="2"/>
+      <c r="H340" s="2"/>
+      <c r="I340" s="2"/>
+      <c r="J340" s="2"/>
+      <c r="K340" s="2"/>
+      <c r="L340" s="2"/>
+      <c r="M340" s="2"/>
+      <c r="N340" s="2"/>
+      <c r="O340" s="2"/>
+      <c r="P340" s="2"/>
+      <c r="Q340" s="2"/>
+      <c r="R340" s="2"/>
+      <c r="S340" s="2"/>
+      <c r="T340" s="2"/>
+      <c r="U340" s="2"/>
+      <c r="V340" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="444">
-    <mergeCell ref="B324:B325"/>
-    <mergeCell ref="C324:C325"/>
-    <mergeCell ref="D324:D325"/>
-    <mergeCell ref="B326:B327"/>
-    <mergeCell ref="C326:C327"/>
-    <mergeCell ref="D326:D327"/>
-    <mergeCell ref="E319:H319"/>
-    <mergeCell ref="I319:L319"/>
-    <mergeCell ref="M319:P319"/>
-    <mergeCell ref="Q319:V319"/>
-    <mergeCell ref="B320:B321"/>
-    <mergeCell ref="C320:C321"/>
-    <mergeCell ref="D320:D321"/>
-    <mergeCell ref="B322:B323"/>
-    <mergeCell ref="C322:C323"/>
-    <mergeCell ref="D322:D323"/>
-    <mergeCell ref="B312:B313"/>
-    <mergeCell ref="C312:C313"/>
-    <mergeCell ref="D312:D313"/>
-    <mergeCell ref="B314:B315"/>
-    <mergeCell ref="C314:C315"/>
-    <mergeCell ref="D314:D315"/>
-    <mergeCell ref="E307:H307"/>
-    <mergeCell ref="I307:L307"/>
-    <mergeCell ref="M307:P307"/>
-    <mergeCell ref="Q307:V307"/>
-    <mergeCell ref="B308:B309"/>
-    <mergeCell ref="C308:C309"/>
-    <mergeCell ref="D308:D309"/>
-    <mergeCell ref="B310:B311"/>
-    <mergeCell ref="C310:C311"/>
-    <mergeCell ref="D310:D311"/>
-    <mergeCell ref="B262:B263"/>
-    <mergeCell ref="C262:C263"/>
-    <mergeCell ref="D262:D263"/>
-    <mergeCell ref="B264:B265"/>
-    <mergeCell ref="C264:C265"/>
-    <mergeCell ref="D264:D265"/>
-    <mergeCell ref="B274:B275"/>
-    <mergeCell ref="C274:C275"/>
-    <mergeCell ref="D274:D275"/>
-    <mergeCell ref="E269:H269"/>
-    <mergeCell ref="I269:L269"/>
-    <mergeCell ref="M269:P269"/>
-    <mergeCell ref="Q269:V269"/>
-    <mergeCell ref="B270:B271"/>
-    <mergeCell ref="C270:C271"/>
-    <mergeCell ref="D270:D271"/>
-    <mergeCell ref="B272:B273"/>
-    <mergeCell ref="E257:H257"/>
-    <mergeCell ref="I257:L257"/>
-    <mergeCell ref="M257:P257"/>
-    <mergeCell ref="Q257:V257"/>
-    <mergeCell ref="B258:B259"/>
-    <mergeCell ref="C258:C259"/>
-    <mergeCell ref="D258:D259"/>
-    <mergeCell ref="B260:B261"/>
-    <mergeCell ref="C260:C261"/>
-    <mergeCell ref="D260:D261"/>
-    <mergeCell ref="B252:B253"/>
-    <mergeCell ref="C252:C253"/>
-    <mergeCell ref="D252:D253"/>
-    <mergeCell ref="Q245:V245"/>
-    <mergeCell ref="B246:B247"/>
-    <mergeCell ref="C246:C247"/>
-    <mergeCell ref="D246:D247"/>
-    <mergeCell ref="B248:B249"/>
-    <mergeCell ref="C248:C249"/>
-    <mergeCell ref="D248:D249"/>
-    <mergeCell ref="B250:B251"/>
-    <mergeCell ref="C250:C251"/>
-    <mergeCell ref="D250:D251"/>
-    <mergeCell ref="B238:B239"/>
-    <mergeCell ref="C238:C239"/>
-    <mergeCell ref="D238:D239"/>
-    <mergeCell ref="B240:B241"/>
-    <mergeCell ref="C240:C241"/>
-    <mergeCell ref="D240:D241"/>
-    <mergeCell ref="E245:H245"/>
-    <mergeCell ref="I245:L245"/>
-    <mergeCell ref="M245:P245"/>
-    <mergeCell ref="E233:H233"/>
-    <mergeCell ref="I233:L233"/>
-    <mergeCell ref="M233:P233"/>
-    <mergeCell ref="Q233:V233"/>
-    <mergeCell ref="B234:B235"/>
-    <mergeCell ref="C234:C235"/>
-    <mergeCell ref="D234:D235"/>
-    <mergeCell ref="B236:B237"/>
-    <mergeCell ref="C236:C237"/>
-    <mergeCell ref="D236:D237"/>
+  <mergeCells count="460">
+    <mergeCell ref="B336:B337"/>
+    <mergeCell ref="C336:C337"/>
+    <mergeCell ref="D336:D337"/>
+    <mergeCell ref="B338:B339"/>
+    <mergeCell ref="C338:C339"/>
+    <mergeCell ref="D338:D339"/>
+    <mergeCell ref="E331:H331"/>
+    <mergeCell ref="I331:L331"/>
+    <mergeCell ref="M331:P331"/>
+    <mergeCell ref="Q331:V331"/>
+    <mergeCell ref="B332:B333"/>
+    <mergeCell ref="C332:C333"/>
+    <mergeCell ref="D332:D333"/>
+    <mergeCell ref="B334:B335"/>
+    <mergeCell ref="C334:C335"/>
+    <mergeCell ref="D334:D335"/>
+    <mergeCell ref="B300:B301"/>
+    <mergeCell ref="C300:C301"/>
+    <mergeCell ref="D300:D301"/>
+    <mergeCell ref="B302:B303"/>
+    <mergeCell ref="C302:C303"/>
+    <mergeCell ref="D302:D303"/>
+    <mergeCell ref="E295:H295"/>
+    <mergeCell ref="I295:L295"/>
+    <mergeCell ref="M295:P295"/>
+    <mergeCell ref="Q295:V295"/>
+    <mergeCell ref="B296:B297"/>
+    <mergeCell ref="C296:C297"/>
+    <mergeCell ref="D296:D297"/>
+    <mergeCell ref="B298:B299"/>
+    <mergeCell ref="C298:C299"/>
+    <mergeCell ref="D298:D299"/>
+    <mergeCell ref="B290:B291"/>
+    <mergeCell ref="C290:C291"/>
+    <mergeCell ref="D290:D291"/>
+    <mergeCell ref="B284:B285"/>
+    <mergeCell ref="C284:C285"/>
+    <mergeCell ref="D284:D285"/>
+    <mergeCell ref="B286:B287"/>
+    <mergeCell ref="C286:C287"/>
+    <mergeCell ref="D286:D287"/>
+    <mergeCell ref="B288:B289"/>
+    <mergeCell ref="C288:C289"/>
+    <mergeCell ref="D288:D289"/>
+    <mergeCell ref="E279:H279"/>
+    <mergeCell ref="I279:L279"/>
+    <mergeCell ref="M279:P279"/>
+    <mergeCell ref="Q279:V279"/>
+    <mergeCell ref="B280:B281"/>
+    <mergeCell ref="C280:C281"/>
+    <mergeCell ref="D280:D281"/>
+    <mergeCell ref="B282:B283"/>
+    <mergeCell ref="C282:C283"/>
+    <mergeCell ref="D282:D283"/>
+    <mergeCell ref="B226:B227"/>
+    <mergeCell ref="C226:C227"/>
+    <mergeCell ref="D226:D227"/>
+    <mergeCell ref="B228:B229"/>
+    <mergeCell ref="C228:C229"/>
+    <mergeCell ref="D228:D229"/>
+    <mergeCell ref="E221:H221"/>
+    <mergeCell ref="I221:L221"/>
+    <mergeCell ref="M221:P221"/>
+    <mergeCell ref="Q221:V221"/>
+    <mergeCell ref="B222:B223"/>
+    <mergeCell ref="C222:C223"/>
+    <mergeCell ref="D222:D223"/>
+    <mergeCell ref="B224:B225"/>
+    <mergeCell ref="C224:C225"/>
+    <mergeCell ref="D224:D225"/>
+    <mergeCell ref="B216:B217"/>
+    <mergeCell ref="C216:C217"/>
+    <mergeCell ref="D216:D217"/>
+    <mergeCell ref="E211:H211"/>
+    <mergeCell ref="I211:L211"/>
+    <mergeCell ref="M211:P211"/>
+    <mergeCell ref="Q211:V211"/>
+    <mergeCell ref="B212:B213"/>
+    <mergeCell ref="C212:C213"/>
+    <mergeCell ref="D212:D213"/>
+    <mergeCell ref="B214:B215"/>
+    <mergeCell ref="C214:C215"/>
+    <mergeCell ref="D214:D215"/>
+    <mergeCell ref="B198:B199"/>
+    <mergeCell ref="C198:C199"/>
+    <mergeCell ref="D198:D199"/>
+    <mergeCell ref="B206:B207"/>
+    <mergeCell ref="C206:C207"/>
+    <mergeCell ref="D206:D207"/>
+    <mergeCell ref="B200:B201"/>
+    <mergeCell ref="C200:C201"/>
+    <mergeCell ref="D200:D201"/>
+    <mergeCell ref="B202:B203"/>
+    <mergeCell ref="C202:C203"/>
+    <mergeCell ref="D202:D203"/>
+    <mergeCell ref="B204:B205"/>
+    <mergeCell ref="C204:C205"/>
+    <mergeCell ref="D204:D205"/>
+    <mergeCell ref="B174:B175"/>
+    <mergeCell ref="C174:C175"/>
+    <mergeCell ref="D174:D175"/>
+    <mergeCell ref="E195:H195"/>
+    <mergeCell ref="I195:L195"/>
+    <mergeCell ref="M195:P195"/>
+    <mergeCell ref="Q195:V195"/>
+    <mergeCell ref="B196:B197"/>
+    <mergeCell ref="C196:C197"/>
+    <mergeCell ref="D196:D197"/>
+    <mergeCell ref="Q183:V183"/>
+    <mergeCell ref="B184:B185"/>
+    <mergeCell ref="C184:C185"/>
+    <mergeCell ref="D184:D185"/>
+    <mergeCell ref="B190:B191"/>
+    <mergeCell ref="C190:C191"/>
+    <mergeCell ref="D190:D191"/>
+    <mergeCell ref="E183:H183"/>
+    <mergeCell ref="I183:L183"/>
+    <mergeCell ref="M183:P183"/>
+    <mergeCell ref="B186:B187"/>
+    <mergeCell ref="C186:C187"/>
+    <mergeCell ref="D186:D187"/>
+    <mergeCell ref="B116:B117"/>
+    <mergeCell ref="C116:C117"/>
+    <mergeCell ref="D116:D117"/>
+    <mergeCell ref="B118:B119"/>
+    <mergeCell ref="C118:C119"/>
+    <mergeCell ref="D118:D119"/>
+    <mergeCell ref="B130:B131"/>
+    <mergeCell ref="C130:C131"/>
+    <mergeCell ref="D130:D131"/>
+    <mergeCell ref="B120:B121"/>
+    <mergeCell ref="C120:C121"/>
+    <mergeCell ref="D120:D121"/>
+    <mergeCell ref="B126:B127"/>
+    <mergeCell ref="C126:C127"/>
+    <mergeCell ref="D126:D127"/>
+    <mergeCell ref="B128:B129"/>
+    <mergeCell ref="C128:C129"/>
+    <mergeCell ref="D128:D129"/>
+    <mergeCell ref="E113:H113"/>
+    <mergeCell ref="I113:L113"/>
+    <mergeCell ref="M113:P113"/>
+    <mergeCell ref="B80:B81"/>
+    <mergeCell ref="C80:C81"/>
+    <mergeCell ref="D80:D81"/>
+    <mergeCell ref="M77:P77"/>
+    <mergeCell ref="Q89:V89"/>
+    <mergeCell ref="M89:P89"/>
+    <mergeCell ref="B94:B95"/>
+    <mergeCell ref="Q113:V113"/>
+    <mergeCell ref="Q77:V77"/>
+    <mergeCell ref="E101:H101"/>
+    <mergeCell ref="I101:L101"/>
+    <mergeCell ref="M101:P101"/>
+    <mergeCell ref="Q101:V101"/>
+    <mergeCell ref="C106:C107"/>
+    <mergeCell ref="D106:D107"/>
+    <mergeCell ref="B108:B109"/>
+    <mergeCell ref="C108:C109"/>
+    <mergeCell ref="D108:D109"/>
+    <mergeCell ref="B114:B115"/>
+    <mergeCell ref="C114:C115"/>
+    <mergeCell ref="D114:D115"/>
+    <mergeCell ref="B70:B71"/>
+    <mergeCell ref="C70:C71"/>
+    <mergeCell ref="D70:D71"/>
+    <mergeCell ref="B72:B73"/>
+    <mergeCell ref="C72:C73"/>
+    <mergeCell ref="D72:D73"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="C78:C79"/>
+    <mergeCell ref="D78:D79"/>
+    <mergeCell ref="C94:C95"/>
+    <mergeCell ref="D94:D95"/>
+    <mergeCell ref="B96:B97"/>
+    <mergeCell ref="C96:C97"/>
+    <mergeCell ref="D96:D97"/>
+    <mergeCell ref="B102:B103"/>
+    <mergeCell ref="C102:C103"/>
+    <mergeCell ref="D102:D103"/>
+    <mergeCell ref="B104:B105"/>
+    <mergeCell ref="C104:C105"/>
+    <mergeCell ref="D104:D105"/>
+    <mergeCell ref="B106:B107"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="C66:C67"/>
+    <mergeCell ref="D66:D67"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="C68:C69"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="E63:H63"/>
+    <mergeCell ref="I63:L63"/>
+    <mergeCell ref="M63:P63"/>
+    <mergeCell ref="Q63:V63"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="D58:D59"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="E49:H49"/>
+    <mergeCell ref="I49:L49"/>
+    <mergeCell ref="M49:P49"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="Q49:V49"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="E37:H37"/>
+    <mergeCell ref="I37:L37"/>
+    <mergeCell ref="M37:P37"/>
+    <mergeCell ref="Q37:V37"/>
+    <mergeCell ref="M24:P24"/>
+    <mergeCell ref="Q24:V24"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E24:H24"/>
+    <mergeCell ref="I24:L24"/>
+    <mergeCell ref="M2:P2"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E13:H13"/>
+    <mergeCell ref="I13:L13"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="Q2:V2"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="M13:P13"/>
+    <mergeCell ref="Q13:V13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="C90:C91"/>
+    <mergeCell ref="D90:D91"/>
+    <mergeCell ref="B92:B93"/>
+    <mergeCell ref="C92:C93"/>
+    <mergeCell ref="D92:D93"/>
+    <mergeCell ref="E77:H77"/>
+    <mergeCell ref="I77:L77"/>
+    <mergeCell ref="B82:B83"/>
+    <mergeCell ref="C82:C83"/>
+    <mergeCell ref="D82:D83"/>
+    <mergeCell ref="B84:B85"/>
+    <mergeCell ref="C84:C85"/>
+    <mergeCell ref="D84:D85"/>
+    <mergeCell ref="E89:H89"/>
+    <mergeCell ref="I89:L89"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="E135:H135"/>
+    <mergeCell ref="I135:L135"/>
+    <mergeCell ref="M135:P135"/>
+    <mergeCell ref="E125:H125"/>
+    <mergeCell ref="I125:L125"/>
+    <mergeCell ref="M125:P125"/>
+    <mergeCell ref="Q135:V135"/>
+    <mergeCell ref="B136:B137"/>
+    <mergeCell ref="C136:C137"/>
+    <mergeCell ref="D136:D137"/>
+    <mergeCell ref="Q125:V125"/>
+    <mergeCell ref="Q159:V159"/>
+    <mergeCell ref="Q171:V171"/>
+    <mergeCell ref="B138:B139"/>
+    <mergeCell ref="C138:C139"/>
+    <mergeCell ref="D138:D139"/>
+    <mergeCell ref="B140:B141"/>
+    <mergeCell ref="C140:C141"/>
+    <mergeCell ref="D140:D141"/>
+    <mergeCell ref="Q147:V147"/>
+    <mergeCell ref="B148:B149"/>
+    <mergeCell ref="C148:C149"/>
+    <mergeCell ref="D148:D149"/>
+    <mergeCell ref="B142:B143"/>
+    <mergeCell ref="C142:C143"/>
+    <mergeCell ref="D142:D143"/>
+    <mergeCell ref="E147:H147"/>
+    <mergeCell ref="I147:L147"/>
+    <mergeCell ref="M147:P147"/>
+    <mergeCell ref="B164:B165"/>
+    <mergeCell ref="C164:C165"/>
+    <mergeCell ref="B150:B151"/>
+    <mergeCell ref="C150:C151"/>
+    <mergeCell ref="D150:D151"/>
+    <mergeCell ref="B152:B153"/>
+    <mergeCell ref="C152:C153"/>
+    <mergeCell ref="D152:D153"/>
+    <mergeCell ref="D164:D165"/>
+    <mergeCell ref="B166:B167"/>
+    <mergeCell ref="C166:C167"/>
+    <mergeCell ref="D166:D167"/>
+    <mergeCell ref="B154:B155"/>
+    <mergeCell ref="C154:C155"/>
+    <mergeCell ref="D154:D155"/>
     <mergeCell ref="E159:H159"/>
     <mergeCell ref="I159:L159"/>
     <mergeCell ref="M159:P159"/>
@@ -27136,335 +27789,99 @@
     <mergeCell ref="E171:H171"/>
     <mergeCell ref="I171:L171"/>
     <mergeCell ref="M171:P171"/>
-    <mergeCell ref="C152:C153"/>
-    <mergeCell ref="D152:D153"/>
-    <mergeCell ref="D164:D165"/>
-    <mergeCell ref="B166:B167"/>
-    <mergeCell ref="C166:C167"/>
-    <mergeCell ref="D166:D167"/>
-    <mergeCell ref="B154:B155"/>
-    <mergeCell ref="C154:C155"/>
-    <mergeCell ref="D154:D155"/>
-    <mergeCell ref="Q159:V159"/>
-    <mergeCell ref="Q171:V171"/>
-    <mergeCell ref="B138:B139"/>
-    <mergeCell ref="C138:C139"/>
-    <mergeCell ref="D138:D139"/>
-    <mergeCell ref="B140:B141"/>
-    <mergeCell ref="C140:C141"/>
-    <mergeCell ref="D140:D141"/>
-    <mergeCell ref="Q147:V147"/>
-    <mergeCell ref="B148:B149"/>
-    <mergeCell ref="C148:C149"/>
-    <mergeCell ref="D148:D149"/>
-    <mergeCell ref="B142:B143"/>
-    <mergeCell ref="C142:C143"/>
-    <mergeCell ref="D142:D143"/>
-    <mergeCell ref="E147:H147"/>
-    <mergeCell ref="I147:L147"/>
-    <mergeCell ref="M147:P147"/>
-    <mergeCell ref="B164:B165"/>
-    <mergeCell ref="C164:C165"/>
-    <mergeCell ref="B150:B151"/>
-    <mergeCell ref="C150:C151"/>
-    <mergeCell ref="D150:D151"/>
-    <mergeCell ref="B152:B153"/>
-    <mergeCell ref="E135:H135"/>
-    <mergeCell ref="I135:L135"/>
-    <mergeCell ref="M135:P135"/>
-    <mergeCell ref="E125:H125"/>
-    <mergeCell ref="I125:L125"/>
-    <mergeCell ref="M125:P125"/>
-    <mergeCell ref="Q135:V135"/>
-    <mergeCell ref="B136:B137"/>
-    <mergeCell ref="C136:C137"/>
-    <mergeCell ref="D136:D137"/>
-    <mergeCell ref="Q125:V125"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="B90:B91"/>
-    <mergeCell ref="C90:C91"/>
-    <mergeCell ref="D90:D91"/>
-    <mergeCell ref="B92:B93"/>
-    <mergeCell ref="C92:C93"/>
-    <mergeCell ref="D92:D93"/>
-    <mergeCell ref="E77:H77"/>
-    <mergeCell ref="I77:L77"/>
-    <mergeCell ref="B82:B83"/>
-    <mergeCell ref="C82:C83"/>
-    <mergeCell ref="D82:D83"/>
-    <mergeCell ref="B84:B85"/>
-    <mergeCell ref="C84:C85"/>
-    <mergeCell ref="D84:D85"/>
-    <mergeCell ref="E89:H89"/>
-    <mergeCell ref="I89:L89"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="M13:P13"/>
-    <mergeCell ref="Q13:V13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="M24:P24"/>
-    <mergeCell ref="Q24:V24"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E24:H24"/>
-    <mergeCell ref="I24:L24"/>
-    <mergeCell ref="M2:P2"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E13:H13"/>
-    <mergeCell ref="I13:L13"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="Q2:V2"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="E37:H37"/>
-    <mergeCell ref="I37:L37"/>
-    <mergeCell ref="M37:P37"/>
-    <mergeCell ref="Q37:V37"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="Q49:V49"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="E49:H49"/>
-    <mergeCell ref="I49:L49"/>
-    <mergeCell ref="M49:P49"/>
-    <mergeCell ref="Q63:V63"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="C58:C59"/>
-    <mergeCell ref="D58:D59"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="C56:C57"/>
-    <mergeCell ref="D56:D57"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="C66:C67"/>
-    <mergeCell ref="D66:D67"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="C68:C69"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="E63:H63"/>
-    <mergeCell ref="I63:L63"/>
-    <mergeCell ref="M63:P63"/>
-    <mergeCell ref="B114:B115"/>
-    <mergeCell ref="C114:C115"/>
-    <mergeCell ref="D114:D115"/>
-    <mergeCell ref="B70:B71"/>
-    <mergeCell ref="C70:C71"/>
-    <mergeCell ref="D70:D71"/>
-    <mergeCell ref="B72:B73"/>
-    <mergeCell ref="C72:C73"/>
-    <mergeCell ref="D72:D73"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="C78:C79"/>
-    <mergeCell ref="D78:D79"/>
-    <mergeCell ref="C94:C95"/>
-    <mergeCell ref="D94:D95"/>
-    <mergeCell ref="B96:B97"/>
-    <mergeCell ref="C96:C97"/>
-    <mergeCell ref="D96:D97"/>
-    <mergeCell ref="B102:B103"/>
-    <mergeCell ref="C102:C103"/>
-    <mergeCell ref="D102:D103"/>
-    <mergeCell ref="B104:B105"/>
-    <mergeCell ref="C104:C105"/>
-    <mergeCell ref="D104:D105"/>
-    <mergeCell ref="B106:B107"/>
-    <mergeCell ref="E113:H113"/>
-    <mergeCell ref="I113:L113"/>
-    <mergeCell ref="M113:P113"/>
-    <mergeCell ref="B80:B81"/>
-    <mergeCell ref="C80:C81"/>
-    <mergeCell ref="D80:D81"/>
-    <mergeCell ref="M77:P77"/>
-    <mergeCell ref="Q89:V89"/>
-    <mergeCell ref="M89:P89"/>
-    <mergeCell ref="B94:B95"/>
-    <mergeCell ref="Q113:V113"/>
-    <mergeCell ref="Q77:V77"/>
-    <mergeCell ref="E101:H101"/>
-    <mergeCell ref="I101:L101"/>
-    <mergeCell ref="M101:P101"/>
-    <mergeCell ref="Q101:V101"/>
-    <mergeCell ref="C106:C107"/>
-    <mergeCell ref="D106:D107"/>
-    <mergeCell ref="B108:B109"/>
-    <mergeCell ref="C108:C109"/>
-    <mergeCell ref="D108:D109"/>
-    <mergeCell ref="B116:B117"/>
-    <mergeCell ref="C116:C117"/>
-    <mergeCell ref="D116:D117"/>
-    <mergeCell ref="B118:B119"/>
-    <mergeCell ref="C118:C119"/>
-    <mergeCell ref="D118:D119"/>
-    <mergeCell ref="B130:B131"/>
-    <mergeCell ref="C130:C131"/>
-    <mergeCell ref="D130:D131"/>
-    <mergeCell ref="B120:B121"/>
-    <mergeCell ref="C120:C121"/>
-    <mergeCell ref="D120:D121"/>
-    <mergeCell ref="B126:B127"/>
-    <mergeCell ref="C126:C127"/>
-    <mergeCell ref="D126:D127"/>
-    <mergeCell ref="B128:B129"/>
-    <mergeCell ref="C128:C129"/>
-    <mergeCell ref="D128:D129"/>
-    <mergeCell ref="B174:B175"/>
-    <mergeCell ref="C174:C175"/>
-    <mergeCell ref="D174:D175"/>
-    <mergeCell ref="E195:H195"/>
-    <mergeCell ref="I195:L195"/>
-    <mergeCell ref="M195:P195"/>
-    <mergeCell ref="Q195:V195"/>
-    <mergeCell ref="B196:B197"/>
-    <mergeCell ref="C196:C197"/>
-    <mergeCell ref="D196:D197"/>
-    <mergeCell ref="Q183:V183"/>
-    <mergeCell ref="B184:B185"/>
-    <mergeCell ref="C184:C185"/>
-    <mergeCell ref="D184:D185"/>
-    <mergeCell ref="B190:B191"/>
-    <mergeCell ref="C190:C191"/>
-    <mergeCell ref="D190:D191"/>
-    <mergeCell ref="E183:H183"/>
-    <mergeCell ref="I183:L183"/>
-    <mergeCell ref="M183:P183"/>
-    <mergeCell ref="B186:B187"/>
-    <mergeCell ref="C186:C187"/>
-    <mergeCell ref="D186:D187"/>
-    <mergeCell ref="B198:B199"/>
-    <mergeCell ref="C198:C199"/>
-    <mergeCell ref="D198:D199"/>
-    <mergeCell ref="B206:B207"/>
-    <mergeCell ref="C206:C207"/>
-    <mergeCell ref="D206:D207"/>
-    <mergeCell ref="B200:B201"/>
-    <mergeCell ref="C200:C201"/>
-    <mergeCell ref="D200:D201"/>
-    <mergeCell ref="B202:B203"/>
-    <mergeCell ref="C202:C203"/>
-    <mergeCell ref="D202:D203"/>
-    <mergeCell ref="B204:B205"/>
-    <mergeCell ref="C204:C205"/>
-    <mergeCell ref="D204:D205"/>
-    <mergeCell ref="E211:H211"/>
-    <mergeCell ref="I211:L211"/>
-    <mergeCell ref="M211:P211"/>
-    <mergeCell ref="Q211:V211"/>
-    <mergeCell ref="B212:B213"/>
-    <mergeCell ref="C212:C213"/>
-    <mergeCell ref="D212:D213"/>
-    <mergeCell ref="B214:B215"/>
-    <mergeCell ref="C214:C215"/>
-    <mergeCell ref="D214:D215"/>
-    <mergeCell ref="Q221:V221"/>
-    <mergeCell ref="B222:B223"/>
-    <mergeCell ref="C222:C223"/>
-    <mergeCell ref="D222:D223"/>
-    <mergeCell ref="B224:B225"/>
-    <mergeCell ref="C224:C225"/>
-    <mergeCell ref="D224:D225"/>
-    <mergeCell ref="B216:B217"/>
-    <mergeCell ref="C216:C217"/>
-    <mergeCell ref="D216:D217"/>
-    <mergeCell ref="B226:B227"/>
-    <mergeCell ref="C226:C227"/>
-    <mergeCell ref="D226:D227"/>
-    <mergeCell ref="B228:B229"/>
-    <mergeCell ref="C228:C229"/>
-    <mergeCell ref="D228:D229"/>
-    <mergeCell ref="E221:H221"/>
-    <mergeCell ref="I221:L221"/>
-    <mergeCell ref="M221:P221"/>
+    <mergeCell ref="E233:H233"/>
+    <mergeCell ref="I233:L233"/>
+    <mergeCell ref="M233:P233"/>
+    <mergeCell ref="Q233:V233"/>
+    <mergeCell ref="B234:B235"/>
+    <mergeCell ref="C234:C235"/>
+    <mergeCell ref="D234:D235"/>
+    <mergeCell ref="B236:B237"/>
+    <mergeCell ref="C236:C237"/>
+    <mergeCell ref="D236:D237"/>
+    <mergeCell ref="B238:B239"/>
+    <mergeCell ref="C238:C239"/>
+    <mergeCell ref="D238:D239"/>
+    <mergeCell ref="B240:B241"/>
+    <mergeCell ref="C240:C241"/>
+    <mergeCell ref="D240:D241"/>
+    <mergeCell ref="E245:H245"/>
+    <mergeCell ref="I245:L245"/>
+    <mergeCell ref="M245:P245"/>
+    <mergeCell ref="B252:B253"/>
+    <mergeCell ref="C252:C253"/>
+    <mergeCell ref="D252:D253"/>
+    <mergeCell ref="Q245:V245"/>
+    <mergeCell ref="B246:B247"/>
+    <mergeCell ref="C246:C247"/>
+    <mergeCell ref="D246:D247"/>
+    <mergeCell ref="B248:B249"/>
+    <mergeCell ref="C248:C249"/>
+    <mergeCell ref="D248:D249"/>
+    <mergeCell ref="B250:B251"/>
+    <mergeCell ref="C250:C251"/>
+    <mergeCell ref="D250:D251"/>
+    <mergeCell ref="E269:H269"/>
+    <mergeCell ref="I269:L269"/>
+    <mergeCell ref="M269:P269"/>
+    <mergeCell ref="Q269:V269"/>
+    <mergeCell ref="B270:B271"/>
+    <mergeCell ref="C270:C271"/>
+    <mergeCell ref="D270:D271"/>
+    <mergeCell ref="B272:B273"/>
+    <mergeCell ref="E257:H257"/>
+    <mergeCell ref="I257:L257"/>
+    <mergeCell ref="M257:P257"/>
+    <mergeCell ref="Q257:V257"/>
+    <mergeCell ref="B258:B259"/>
+    <mergeCell ref="C258:C259"/>
+    <mergeCell ref="D258:D259"/>
+    <mergeCell ref="B260:B261"/>
+    <mergeCell ref="C260:C261"/>
+    <mergeCell ref="D260:D261"/>
     <mergeCell ref="C272:C273"/>
     <mergeCell ref="D272:D273"/>
-    <mergeCell ref="E279:H279"/>
-    <mergeCell ref="I279:L279"/>
-    <mergeCell ref="M279:P279"/>
-    <mergeCell ref="Q279:V279"/>
-    <mergeCell ref="B280:B281"/>
-    <mergeCell ref="C280:C281"/>
-    <mergeCell ref="D280:D281"/>
-    <mergeCell ref="B282:B283"/>
-    <mergeCell ref="C282:C283"/>
-    <mergeCell ref="D282:D283"/>
-    <mergeCell ref="B284:B285"/>
-    <mergeCell ref="C284:C285"/>
-    <mergeCell ref="D284:D285"/>
-    <mergeCell ref="B286:B287"/>
-    <mergeCell ref="C286:C287"/>
-    <mergeCell ref="D286:D287"/>
-    <mergeCell ref="B288:B289"/>
-    <mergeCell ref="C288:C289"/>
-    <mergeCell ref="D288:D289"/>
-    <mergeCell ref="Q295:V295"/>
-    <mergeCell ref="B296:B297"/>
-    <mergeCell ref="C296:C297"/>
-    <mergeCell ref="D296:D297"/>
-    <mergeCell ref="B298:B299"/>
-    <mergeCell ref="C298:C299"/>
-    <mergeCell ref="D298:D299"/>
-    <mergeCell ref="B290:B291"/>
-    <mergeCell ref="C290:C291"/>
-    <mergeCell ref="D290:D291"/>
-    <mergeCell ref="B300:B301"/>
-    <mergeCell ref="C300:C301"/>
-    <mergeCell ref="D300:D301"/>
-    <mergeCell ref="B302:B303"/>
-    <mergeCell ref="C302:C303"/>
-    <mergeCell ref="D302:D303"/>
-    <mergeCell ref="E295:H295"/>
-    <mergeCell ref="I295:L295"/>
-    <mergeCell ref="M295:P295"/>
+    <mergeCell ref="B262:B263"/>
+    <mergeCell ref="C262:C263"/>
+    <mergeCell ref="D262:D263"/>
+    <mergeCell ref="B264:B265"/>
+    <mergeCell ref="C264:C265"/>
+    <mergeCell ref="D264:D265"/>
+    <mergeCell ref="B274:B275"/>
+    <mergeCell ref="C274:C275"/>
+    <mergeCell ref="D274:D275"/>
+    <mergeCell ref="E307:H307"/>
+    <mergeCell ref="I307:L307"/>
+    <mergeCell ref="M307:P307"/>
+    <mergeCell ref="Q307:V307"/>
+    <mergeCell ref="B308:B309"/>
+    <mergeCell ref="C308:C309"/>
+    <mergeCell ref="D308:D309"/>
+    <mergeCell ref="B310:B311"/>
+    <mergeCell ref="C310:C311"/>
+    <mergeCell ref="D310:D311"/>
+    <mergeCell ref="Q319:V319"/>
+    <mergeCell ref="B320:B321"/>
+    <mergeCell ref="C320:C321"/>
+    <mergeCell ref="D320:D321"/>
+    <mergeCell ref="B322:B323"/>
+    <mergeCell ref="C322:C323"/>
+    <mergeCell ref="D322:D323"/>
+    <mergeCell ref="B312:B313"/>
+    <mergeCell ref="C312:C313"/>
+    <mergeCell ref="D312:D313"/>
+    <mergeCell ref="B314:B315"/>
+    <mergeCell ref="C314:C315"/>
+    <mergeCell ref="D314:D315"/>
+    <mergeCell ref="B324:B325"/>
+    <mergeCell ref="C324:C325"/>
+    <mergeCell ref="D324:D325"/>
+    <mergeCell ref="B326:B327"/>
+    <mergeCell ref="C326:C327"/>
+    <mergeCell ref="D326:D327"/>
+    <mergeCell ref="E319:H319"/>
+    <mergeCell ref="I319:L319"/>
+    <mergeCell ref="M319:P319"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.74805557727813721" right="0.74805557727813721" top="0.98430556058883667" bottom="0.98430556058883667" header="0.51138889789581299" footer="0.51138889789581299"/>
@@ -27506,23 +27923,23 @@
     <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="D2" s="15">
         <f>SUM(D4:D95)</f>
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="E2" s="15">
         <f>SUM(E4:E95)</f>
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="F2" s="15">
         <f>SUM(F4:F95)</f>
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="G2" s="15">
         <f>SUM(G4:G95)</f>
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="H2" s="15">
         <f>SUM(H4:H95)</f>
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.25">
@@ -27601,7 +28018,7 @@
       </c>
       <c r="C4" s="2">
         <f>((D4+E4+G4+H4)*0.2)+(F4*0.3)</f>
-        <v>2.2000000000000002</v>
+        <v>2.6</v>
       </c>
       <c r="D4" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B4)</f>
@@ -27609,7 +28026,7 @@
       </c>
       <c r="E4" s="14">
         <f>COUNTIF(경기기록Sheet!$I:$L,B4)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F4" s="14">
         <f>COUNTIF(경기기록Sheet!$M:$P,B4)</f>
@@ -27625,7 +28042,7 @@
       </c>
       <c r="I4" s="14">
         <f>SUM(D4:H4)</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J4" s="15"/>
       <c r="K4" s="2">
@@ -27664,7 +28081,7 @@
       </c>
       <c r="U4" s="56">
         <f t="shared" ref="U4:U14" si="4">VLOOKUP(T4,$B$4:$H$133,7,FALSE)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
@@ -27727,14 +28144,14 @@
       </c>
       <c r="Q5" s="23">
         <f t="shared" si="2"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R5" s="35" t="s">
         <v>230</v>
       </c>
       <c r="S5" s="55">
         <f t="shared" si="3"/>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="T5" s="36" t="s">
         <v>228</v>
@@ -27790,10 +28207,10 @@
       </c>
       <c r="M6" s="21">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N6" s="33" t="s">
-        <v>356</v>
+        <v>50</v>
       </c>
       <c r="O6" s="22">
         <f t="shared" si="1"/>
@@ -27863,18 +28280,18 @@
         <v>4</v>
       </c>
       <c r="L7" s="32" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="M7" s="21">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="N7" s="33" t="s">
-        <v>221</v>
+        <v>356</v>
       </c>
       <c r="O7" s="22">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P7" s="34" t="s">
         <v>298</v>
@@ -27884,18 +28301,18 @@
         <v>8</v>
       </c>
       <c r="R7" s="35" t="s">
-        <v>359</v>
+        <v>232</v>
       </c>
       <c r="S7" s="55">
         <f t="shared" si="3"/>
         <v>16</v>
       </c>
       <c r="T7" s="36" t="s">
-        <v>352</v>
+        <v>181</v>
       </c>
       <c r="U7" s="56">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.25">
@@ -27940,18 +28357,18 @@
         <v>5</v>
       </c>
       <c r="L8" s="32" t="s">
-        <v>352</v>
+        <v>221</v>
       </c>
       <c r="M8" s="21">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="N8" s="33" t="s">
-        <v>50</v>
+        <v>221</v>
       </c>
       <c r="O8" s="22">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P8" s="34" t="s">
         <v>53</v>
@@ -27961,14 +28378,14 @@
         <v>8</v>
       </c>
       <c r="R8" s="35" t="s">
-        <v>232</v>
+        <v>62</v>
       </c>
       <c r="S8" s="55">
         <f t="shared" si="3"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T8" s="36" t="s">
-        <v>353</v>
+        <v>311</v>
       </c>
       <c r="U8" s="56">
         <f t="shared" si="4"/>
@@ -28017,7 +28434,7 @@
         <v>6</v>
       </c>
       <c r="L9" s="32" t="s">
-        <v>231</v>
+        <v>352</v>
       </c>
       <c r="M9" s="21">
         <f t="shared" si="0"/>
@@ -28038,11 +28455,11 @@
         <v>8</v>
       </c>
       <c r="R9" s="35" t="s">
-        <v>62</v>
+        <v>359</v>
       </c>
       <c r="S9" s="55">
         <f t="shared" si="3"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T9" s="36" t="s">
         <v>396</v>
@@ -28192,7 +28609,7 @@
         <v>7</v>
       </c>
       <c r="R11" s="35" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="S11" s="55">
         <f t="shared" si="3"/>
@@ -28248,11 +28665,11 @@
         <v>9</v>
       </c>
       <c r="L12" s="32" t="s">
-        <v>304</v>
+        <v>406</v>
       </c>
       <c r="M12" s="21">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N12" s="33" t="s">
         <v>397</v>
@@ -28269,11 +28686,11 @@
         <v>6</v>
       </c>
       <c r="R12" s="35" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="S12" s="55">
         <f t="shared" si="3"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T12" s="36" t="s">
         <v>360</v>
@@ -28325,11 +28742,11 @@
         <v>10</v>
       </c>
       <c r="L13" s="32" t="s">
-        <v>406</v>
+        <v>304</v>
       </c>
       <c r="M13" s="21">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N13" s="33" t="s">
         <v>352</v>
@@ -28346,11 +28763,11 @@
         <v>5</v>
       </c>
       <c r="R13" s="35" t="s">
-        <v>34</v>
+        <v>360</v>
       </c>
       <c r="S13" s="55">
         <f t="shared" si="3"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T13" s="36" t="s">
         <v>359</v>
@@ -28423,11 +28840,11 @@
         <v>5</v>
       </c>
       <c r="R14" s="55" t="s">
-        <v>221</v>
+        <v>34</v>
       </c>
       <c r="S14" s="55">
         <f t="shared" si="3"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T14" s="36" t="s">
         <v>229</v>
@@ -28500,7 +28917,7 @@
         <v>5</v>
       </c>
       <c r="R15" s="55" t="s">
-        <v>241</v>
+        <v>221</v>
       </c>
       <c r="S15" s="55">
         <f t="shared" si="3"/>
@@ -28564,15 +28981,10 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="P16" s="23" t="s">
-        <v>223</v>
-      </c>
-      <c r="Q16" s="23">
-        <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
+      <c r="P16" s="23"/>
+      <c r="Q16" s="23"/>
       <c r="R16" s="55" t="s">
-        <v>360</v>
+        <v>241</v>
       </c>
       <c r="S16" s="55">
         <f t="shared" si="3"/>
@@ -28631,9 +29043,7 @@
       </c>
       <c r="N17" s="22"/>
       <c r="O17" s="22"/>
-      <c r="P17" s="23" t="s">
-        <v>316</v>
-      </c>
+      <c r="P17" s="23"/>
       <c r="Q17" s="23"/>
       <c r="R17" s="55" t="s">
         <v>67</v>
@@ -28697,13 +29107,8 @@
       <c r="O18" s="22"/>
       <c r="P18" s="23"/>
       <c r="Q18" s="23"/>
-      <c r="R18" s="55" t="s">
-        <v>229</v>
-      </c>
-      <c r="S18" s="55">
-        <f t="shared" si="3"/>
-        <v>7</v>
-      </c>
+      <c r="R18" s="55"/>
+      <c r="S18" s="55"/>
       <c r="T18" s="56"/>
       <c r="U18" s="56"/>
     </row>
@@ -28913,7 +29318,7 @@
       </c>
       <c r="C24" s="2">
         <f>((D24+E24+G24+H24)*0.2)+(F24*0.3)</f>
-        <v>1.1000000000000001</v>
+        <v>1.3</v>
       </c>
       <c r="D24" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B24)</f>
@@ -28933,11 +29338,11 @@
       </c>
       <c r="H24" s="14">
         <f>COUNTIF(경기기록Sheet!$V:$V,B24)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" s="14">
         <f>SUM(D24:H24)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J24" s="15"/>
     </row>
@@ -29615,7 +30020,7 @@
       </c>
       <c r="C42" s="2">
         <f>((D42+E42+G42+H42)*0.2)+(F42*0.3)</f>
-        <v>4.6000000000000005</v>
+        <v>4.8000000000000007</v>
       </c>
       <c r="D42" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B42)</f>
@@ -29635,11 +30040,11 @@
       </c>
       <c r="H42" s="14">
         <f>COUNTIF(경기기록Sheet!$V:$V,B42)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I42" s="14">
         <f>SUM(D42:H42)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J42" s="15"/>
     </row>
@@ -29693,19 +30098,19 @@
       </c>
       <c r="C44" s="2">
         <f>((D44+E44+G44+H44)*0.2)+(F44*0.3)</f>
-        <v>2.4</v>
+        <v>3.6000000000000005</v>
       </c>
       <c r="D44" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B44)</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E44" s="14">
         <f>COUNTIF(경기기록Sheet!$I:$L,B44)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F44" s="14">
         <f>COUNTIF(경기기록Sheet!$M:$P,B44)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G44" s="14">
         <f>COUNTIF(경기기록Sheet!$Q:$U,B44)</f>
@@ -29717,7 +30122,7 @@
       </c>
       <c r="I44" s="14">
         <f>SUM(D44:H44)</f>
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="J44" s="15"/>
     </row>
@@ -29771,7 +30176,7 @@
       </c>
       <c r="C46" s="2">
         <f>((D46+E46+G46+H46)*0.2)+(F46*0.3)</f>
-        <v>3.4000000000000004</v>
+        <v>3.6</v>
       </c>
       <c r="D46" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B46)</f>
@@ -29787,7 +30192,7 @@
       </c>
       <c r="G46" s="14">
         <f>COUNTIF(경기기록Sheet!$Q:$U,B46)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H46" s="14">
         <f>COUNTIF(경기기록Sheet!$V:$V,B46)</f>
@@ -29795,7 +30200,7 @@
       </c>
       <c r="I46" s="14">
         <f>SUM(D46:H46)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J46" s="15"/>
     </row>
@@ -29810,7 +30215,7 @@
       </c>
       <c r="C47" s="2">
         <f>((D47+E47+G47+H47)*0.2)+(F47*0.3)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D47" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B47)</f>
@@ -29822,11 +30227,11 @@
       </c>
       <c r="F47" s="14">
         <f>COUNTIF(경기기록Sheet!$M:$P,B47)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G47" s="14">
         <f>COUNTIF(경기기록Sheet!$Q:$U,B47)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H47" s="14">
         <f>COUNTIF(경기기록Sheet!$V:$V,B47)</f>
@@ -29834,7 +30239,7 @@
       </c>
       <c r="I47" s="14">
         <f>SUM(D47:H47)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J47" s="15"/>
     </row>
@@ -30200,7 +30605,7 @@
       </c>
       <c r="C57" s="2">
         <f>((D57+E57+G57+H57)*0.2)+(F57*0.3)</f>
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="D57" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B57)</f>
@@ -30212,7 +30617,7 @@
       </c>
       <c r="F57" s="14">
         <f>COUNTIF(경기기록Sheet!$M:$P,B57)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G57" s="14">
         <f>COUNTIF(경기기록Sheet!$Q:$U,B57)</f>
@@ -30224,7 +30629,7 @@
       </c>
       <c r="I57" s="14">
         <f>SUM(D57:H57)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J57" s="15"/>
     </row>
@@ -30317,7 +30722,7 @@
       </c>
       <c r="C60" s="2">
         <f>((D60+E60+G60+H60)*0.2)+(F60*0.3)</f>
-        <v>0.60000000000000009</v>
+        <v>0.8</v>
       </c>
       <c r="D60" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B60)</f>
@@ -30333,7 +30738,7 @@
       </c>
       <c r="G60" s="14">
         <f>COUNTIF(경기기록Sheet!$Q:$U,B60)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H60" s="14">
         <f>COUNTIF(경기기록Sheet!$V:$V,B60)</f>
@@ -30341,7 +30746,7 @@
       </c>
       <c r="I60" s="14">
         <f>SUM(D60:H60)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J60" s="15"/>
     </row>
@@ -30707,7 +31112,7 @@
       </c>
       <c r="C70" s="2">
         <f>((D70+E70+G70+H70)*0.2)+(F70*0.3)</f>
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="D70" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B70)</f>
@@ -30715,7 +31120,7 @@
       </c>
       <c r="E70" s="14">
         <f>COUNTIF(경기기록Sheet!$I:$L,B70)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F70" s="14">
         <f>COUNTIF(경기기록Sheet!$M:$P,B70)</f>
@@ -30731,7 +31136,7 @@
       </c>
       <c r="I70" s="14">
         <f>SUM(D70:H70)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J70" s="15"/>
     </row>
@@ -30863,7 +31268,7 @@
       </c>
       <c r="C74" s="2">
         <f>((D74+E74+G74+H74)*0.2)+(F74*0.3)</f>
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="D74" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B74)</f>
@@ -30879,7 +31284,7 @@
       </c>
       <c r="G74" s="14">
         <f>COUNTIF(경기기록Sheet!$Q:$U,B74)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H74" s="14">
         <f>COUNTIF(경기기록Sheet!$V:$V,B74)</f>
@@ -30887,7 +31292,7 @@
       </c>
       <c r="I74" s="14">
         <f>SUM(D74:H74)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J74" s="15"/>
     </row>
@@ -31136,7 +31541,7 @@
       </c>
       <c r="C81" s="2">
         <f>((D81+E81+G81+H81)*0.2)+(F81*0.3)</f>
-        <v>2.6</v>
+        <v>3</v>
       </c>
       <c r="D81" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B81)</f>
@@ -31152,7 +31557,7 @@
       </c>
       <c r="G81" s="14">
         <f>COUNTIF(경기기록Sheet!$Q:$U,B81)</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H81" s="14">
         <f>COUNTIF(경기기록Sheet!$V:$V,B81)</f>
@@ -31160,7 +31565,7 @@
       </c>
       <c r="I81" s="14">
         <f>SUM(D81:H81)</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J81" s="15"/>
     </row>
@@ -31214,7 +31619,7 @@
       </c>
       <c r="C83" s="2">
         <f>((D83+E83+G83+H83)*0.2)+(F83*0.3)</f>
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="D83" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B83)</f>
@@ -31230,7 +31635,7 @@
       </c>
       <c r="G83" s="14">
         <f>COUNTIF(경기기록Sheet!$Q:$U,B83)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H83" s="14">
         <f>COUNTIF(경기기록Sheet!$V:$V,B83)</f>
@@ -31238,7 +31643,7 @@
       </c>
       <c r="I83" s="14">
         <f>SUM(D83:H83)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J83" s="15"/>
     </row>
@@ -31643,11 +32048,11 @@
       </c>
       <c r="C94" s="2">
         <f>((D94+E94+G94+H94)*0.2)+(F94*0.3)</f>
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="D94" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B94)</f>
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E94" s="14">
         <f>COUNTIF(경기기록Sheet!$I:$L,B94)</f>
@@ -31667,7 +32072,7 @@
       </c>
       <c r="I94" s="14">
         <f>SUM(D94:H94)</f>
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="J94" s="15"/>
     </row>
@@ -31877,7 +32282,7 @@
       </c>
       <c r="C100" s="2">
         <f>((D100+E100+G100+H100)*0.2)+(F100*0.3)</f>
-        <v>5.6000000000000005</v>
+        <v>5.8000000000000007</v>
       </c>
       <c r="D100" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B100)</f>
@@ -31893,7 +32298,7 @@
       </c>
       <c r="G100" s="14">
         <f>COUNTIF(경기기록Sheet!$Q:$U,B100)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H100" s="14">
         <f>COUNTIF(경기기록Sheet!$V:$V,B100)</f>
@@ -31901,7 +32306,7 @@
       </c>
       <c r="I100" s="14">
         <f>SUM(D100:H100)</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J100" s="15"/>
     </row>
@@ -31916,11 +32321,11 @@
       </c>
       <c r="C101" s="2">
         <f>((D101+E101+G101+H101)*0.2)+(F101*0.3)</f>
-        <v>4.2</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="D101" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B101)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E101" s="14">
         <f>COUNTIF(경기기록Sheet!$I:$L,B101)</f>
@@ -31940,7 +32345,7 @@
       </c>
       <c r="I101" s="14">
         <f>SUM(D101:H101)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J101" s="15"/>
     </row>
@@ -31955,11 +32360,11 @@
       </c>
       <c r="C102" s="2">
         <f>((D102+E102+G102+H102)*0.2)+(F102*0.3)</f>
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="D102" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B102)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E102" s="14">
         <f>COUNTIF(경기기록Sheet!$I:$L,B102)</f>
@@ -31979,7 +32384,7 @@
       </c>
       <c r="I102" s="14">
         <f>SUM(D102:H102)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J102" s="15"/>
     </row>
@@ -31994,7 +32399,7 @@
       </c>
       <c r="C103" s="2">
         <f>((D103+E103+G103+H103)*0.2)+(F103*0.3)</f>
-        <v>6.7</v>
+        <v>7</v>
       </c>
       <c r="D103" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B103)</f>
@@ -32006,7 +32411,7 @@
       </c>
       <c r="F103" s="14">
         <f>COUNTIF(경기기록Sheet!$M:$P,B103)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G103" s="14">
         <f>COUNTIF(경기기록Sheet!$Q:$U,B103)</f>
@@ -32018,7 +32423,7 @@
       </c>
       <c r="I103" s="14">
         <f>SUM(D103:H103)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J103" s="15"/>
     </row>
@@ -32033,7 +32438,7 @@
       </c>
       <c r="C104" s="2">
         <f>((D104+E104+G104+H104)*0.2)+(F104*0.3)</f>
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="D104" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B104)</f>
@@ -32049,7 +32454,7 @@
       </c>
       <c r="G104" s="14">
         <f>COUNTIF(경기기록Sheet!$Q:$U,B104)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H104" s="14">
         <f>COUNTIF(경기기록Sheet!$V:$V,B104)</f>
@@ -32057,7 +32462,7 @@
       </c>
       <c r="I104" s="14">
         <f>SUM(D104:H104)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J104" s="15"/>
     </row>
@@ -32680,7 +33085,7 @@
       </c>
       <c r="C121" s="2">
         <f>((D121+E121+G121+H121)*0.2)+(F121*0.3)</f>
-        <v>4.2</v>
+        <v>4.8000000000000007</v>
       </c>
       <c r="D121" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B121)</f>
@@ -32688,7 +33093,7 @@
       </c>
       <c r="E121" s="14">
         <f>COUNTIF(경기기록Sheet!$I:$L,B121)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F121" s="14">
         <f>COUNTIF(경기기록Sheet!$M:$P,B121)</f>
@@ -32696,15 +33101,15 @@
       </c>
       <c r="G121" s="14">
         <f>COUNTIF(경기기록Sheet!$Q:$U,B121)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H121" s="14">
         <f>COUNTIF(경기기록Sheet!$V:$V,B121)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I121" s="14">
         <f>SUM(D121:H121)</f>
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
@@ -32718,15 +33123,15 @@
       </c>
       <c r="C122" s="2">
         <f>((D122+E122+G122+H122)*0.2)+(F122*0.3)</f>
-        <v>0.8</v>
+        <v>1.6</v>
       </c>
       <c r="D122" s="14">
         <f>COUNTIF(경기기록Sheet!$E:$H,B122)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E122" s="14">
         <f>COUNTIF(경기기록Sheet!$I:$L,B122)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F122" s="14">
         <f>COUNTIF(경기기록Sheet!$M:$P,B122)</f>
@@ -32734,7 +33139,7 @@
       </c>
       <c r="G122" s="14">
         <f>COUNTIF(경기기록Sheet!$Q:$U,B122)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H122" s="14">
         <f>COUNTIF(경기기록Sheet!$V:$V,B122)</f>
@@ -32742,15 +33147,10 @@
       </c>
       <c r="I122" s="14">
         <f>SUM(D122:H122)</f>
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:I3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:I122">
-      <sortCondition ref="A3"/>
-    </sortState>
-  </autoFilter>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="D4:D122">
     <cfRule type="top10" dxfId="9" priority="974" rank="7"/>
@@ -34333,10 +34733,10 @@
       <c r="G2" s="47" t="s">
         <v>328</v>
       </c>
-      <c r="I2" s="99" t="s">
+      <c r="I2" s="94" t="s">
         <v>248</v>
       </c>
-      <c r="J2" s="99"/>
+      <c r="J2" s="94"/>
       <c r="K2" s="65" t="s">
         <v>276</v>
       </c>
@@ -34361,7 +34761,7 @@
       </c>
     </row>
     <row r="3" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B3" s="100" t="s">
+      <c r="B3" s="93" t="s">
         <v>334</v>
       </c>
       <c r="C3" s="72">
@@ -34424,7 +34824,7 @@
       </c>
       <c r="E4" s="62">
         <f>VLOOKUP(D4,종합Sheet!$B$3:$I$121,8,0)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F4" s="70" t="s">
         <v>224</v>
@@ -34500,14 +34900,14 @@
       </c>
       <c r="Q5" s="62">
         <f>VLOOKUP(P5,종합Sheet!$B$3:$I$121,8,0)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R5" s="62" t="s">
         <v>304</v>
       </c>
       <c r="S5" s="63">
         <f>VLOOKUP(R5,종합Sheet!$B$3:$I$121,7,0)</f>
-        <v>30.7</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.25">
@@ -34520,14 +34920,14 @@
       </c>
       <c r="E6" s="47">
         <f>VLOOKUP(D6,종합Sheet!$B$3:$I$121,8,0)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F6" s="70" t="s">
         <v>232</v>
       </c>
       <c r="G6" s="61">
         <f>VLOOKUP(F6,종합Sheet!$B$3:$I$121,7,0)</f>
-        <v>21.4</v>
+        <v>22.6</v>
       </c>
       <c r="I6" s="96"/>
       <c r="J6" s="66">
@@ -34548,14 +34948,14 @@
       </c>
       <c r="Q6" s="69">
         <f>VLOOKUP(P6,종합Sheet!$B$3:$I$121,8,0)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="R6" s="65" t="s">
         <v>230</v>
       </c>
       <c r="S6" s="71">
         <f>VLOOKUP(R6,종합Sheet!$B$3:$I$121,7,0)</f>
-        <v>22.6</v>
+        <v>23.8</v>
       </c>
     </row>
     <row r="7" spans="2:19" x14ac:dyDescent="0.25">
@@ -34568,16 +34968,16 @@
       </c>
       <c r="E7" s="47">
         <f>VLOOKUP(D7,종합Sheet!$B$3:$I$121,8,0)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F7" s="70" t="s">
         <v>304</v>
       </c>
       <c r="G7" s="61">
         <f>VLOOKUP(F7,종합Sheet!$B$3:$I$121,7,0)</f>
-        <v>30.7</v>
-      </c>
-      <c r="I7" s="97"/>
+        <v>32</v>
+      </c>
+      <c r="I7" s="98"/>
       <c r="J7" s="66">
         <v>5</v>
       </c>
@@ -34623,7 +35023,7 @@
       </c>
       <c r="G8" s="63">
         <f>VLOOKUP(F8,종합Sheet!$B$3:$I$121,7,0)</f>
-        <v>27.2</v>
+        <v>28.6</v>
       </c>
       <c r="N8" s="86"/>
       <c r="O8" s="48">
@@ -34661,12 +35061,12 @@
       </c>
       <c r="G9" s="61">
         <f>VLOOKUP(F9,종합Sheet!$B$3:$I$121,7,0)</f>
-        <v>17</v>
-      </c>
-      <c r="I9" s="99" t="s">
+        <v>18</v>
+      </c>
+      <c r="I9" s="94" t="s">
         <v>248</v>
       </c>
-      <c r="J9" s="99"/>
+      <c r="J9" s="94"/>
       <c r="K9" s="65" t="s">
         <v>276</v>
       </c>
@@ -34682,7 +35082,7 @@
       </c>
       <c r="Q9" s="69">
         <f>VLOOKUP(P9,종합Sheet!$B$3:$I$121,8,0)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R9" s="65" t="s">
         <v>309</v>
@@ -34702,14 +35102,14 @@
       </c>
       <c r="E10" s="64">
         <f>VLOOKUP(D10,종합Sheet!$B$3:$I$121,8,0)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F10" s="70" t="s">
         <v>53</v>
       </c>
       <c r="G10" s="61">
         <f>VLOOKUP(F10,종합Sheet!$B$3:$I$121,7,0)</f>
-        <v>18.600000000000001</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="I10" s="95" t="s">
         <v>330</v>
@@ -34739,7 +35139,7 @@
       </c>
       <c r="S10" s="71">
         <f>VLOOKUP(R10,종합Sheet!$B$3:$I$121,7,0)</f>
-        <v>15</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="11" spans="2:19" x14ac:dyDescent="0.25">
@@ -34752,7 +35152,7 @@
       </c>
       <c r="E11" s="65">
         <f>VLOOKUP(D11,종합Sheet!$B$3:$I$121,8,0)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F11" s="70" t="s">
         <v>48</v>
@@ -34819,7 +35219,7 @@
       <c r="L12" s="65">
         <v>8</v>
       </c>
-      <c r="N12" s="98"/>
+      <c r="N12" s="101"/>
       <c r="O12" s="48">
         <v>10</v>
       </c>
@@ -34848,7 +35248,7 @@
       </c>
       <c r="E13" s="65">
         <f>VLOOKUP(D13,종합Sheet!$B$3:$I$121,8,0)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F13" s="70" t="s">
         <v>241</v>
@@ -34884,16 +35284,16 @@
       </c>
       <c r="E14" s="65">
         <f>VLOOKUP(D14,종합Sheet!$B$3:$I$121,8,0)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F14" s="70" t="s">
         <v>228</v>
       </c>
       <c r="G14" s="61">
         <f>VLOOKUP(F14,종합Sheet!$B$3:$I$121,7,0)</f>
-        <v>31.6</v>
-      </c>
-      <c r="I14" s="97"/>
+        <v>32.6</v>
+      </c>
+      <c r="I14" s="98"/>
       <c r="J14" s="66">
         <v>5</v>
       </c>
@@ -34946,20 +35346,20 @@
       </c>
       <c r="E16" s="65">
         <f>VLOOKUP(D16,종합Sheet!$B$3:$I$121,8,0)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F16" s="62" t="s">
         <v>230</v>
       </c>
       <c r="G16" s="63">
         <f>VLOOKUP(F16,종합Sheet!$B$3:$I$121,7,0)</f>
-        <v>22.6</v>
+        <v>23.8</v>
       </c>
       <c r="H16" s="37"/>
-      <c r="I16" s="99" t="s">
+      <c r="I16" s="94" t="s">
         <v>248</v>
       </c>
-      <c r="J16" s="99"/>
+      <c r="J16" s="94"/>
       <c r="K16" s="65" t="s">
         <v>276</v>
       </c>
@@ -35020,10 +35420,10 @@
       <c r="U18"/>
     </row>
     <row r="19" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B19" s="99" t="s">
+      <c r="B19" s="94" t="s">
         <v>248</v>
       </c>
-      <c r="C19" s="99"/>
+      <c r="C19" s="94"/>
       <c r="D19" s="65" t="s">
         <v>276</v>
       </c>
@@ -35074,7 +35474,7 @@
       <c r="E21" s="65" t="s">
         <v>337</v>
       </c>
-      <c r="I21" s="97"/>
+      <c r="I21" s="98"/>
       <c r="J21" s="66">
         <v>5</v>
       </c>
@@ -35086,7 +35486,7 @@
       </c>
     </row>
     <row r="22" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="B22" s="101"/>
+      <c r="B22" s="97"/>
       <c r="C22" s="66">
         <v>3</v>
       </c>
@@ -35098,10 +35498,10 @@
       </c>
     </row>
     <row r="23" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="I23" s="93" t="s">
+      <c r="I23" s="99" t="s">
         <v>248</v>
       </c>
-      <c r="J23" s="94"/>
+      <c r="J23" s="100"/>
       <c r="K23" s="65" t="s">
         <v>276</v>
       </c>
@@ -35184,7 +35584,7 @@
       </c>
     </row>
     <row r="30" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="I30" s="97"/>
+      <c r="I30" s="98"/>
       <c r="J30" s="66">
         <v>7</v>
       </c>
@@ -35197,12 +35597,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B3:B17"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:B22"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="I17:I21"/>
     <mergeCell ref="I23:J23"/>
     <mergeCell ref="I24:I30"/>
     <mergeCell ref="N2:O2"/>
@@ -35211,6 +35605,12 @@
     <mergeCell ref="I3:I7"/>
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="I10:I14"/>
+    <mergeCell ref="B3:B17"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="I17:I21"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -35751,11 +36151,11 @@
       </c>
       <c r="G4" s="2">
         <f t="shared" ref="G4:G37" si="2">RANK(H4,$H$4:$H$37,0)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H4" s="6">
         <f>I4+개인기록Sheet!C4</f>
-        <v>5.2</v>
+        <v>5.6</v>
       </c>
       <c r="I4" s="6">
         <f t="shared" ref="I4:I28" si="3">(COUNTIF(J4:CD4,"출전")*1)</f>
@@ -36665,7 +37065,7 @@
       </c>
       <c r="G12" s="2">
         <f t="shared" si="2"/>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H12" s="6">
         <f>I12+개인기록Sheet!C18</f>
@@ -37328,7 +37728,7 @@
       </c>
       <c r="G18" s="2">
         <f t="shared" si="2"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H18" s="6">
         <f>I18+개인기록Sheet!C29</f>
@@ -37446,7 +37846,7 @@
       </c>
       <c r="G19" s="2">
         <f t="shared" si="2"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H19" s="6">
         <f>I19+개인기록Sheet!C34</f>
@@ -37676,11 +38076,11 @@
       </c>
       <c r="G21" s="2">
         <f t="shared" si="2"/>
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="H21" s="6">
         <f>I21+개인기록Sheet!C44</f>
-        <v>4.4000000000000004</v>
+        <v>5.6000000000000005</v>
       </c>
       <c r="I21" s="6">
         <f t="shared" si="3"/>
@@ -37777,7 +38177,7 @@
       </c>
       <c r="D22" s="2">
         <f>VLOOKUP(B22,종합Sheet!$B$4:$F$133,3,0)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E22" s="2">
         <f>VLOOKUP(B22,종합Sheet!$B$4:$F$133,4,0)</f>
@@ -37887,7 +38287,7 @@
       </c>
       <c r="G23" s="2">
         <f t="shared" si="2"/>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H23" s="6">
         <f>I23+개인기록Sheet!C49</f>
@@ -38003,11 +38403,11 @@
       </c>
       <c r="G24" s="2">
         <f t="shared" si="2"/>
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H24" s="6">
         <f>I24+개인기록Sheet!C57</f>
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="I24" s="6">
         <f t="shared" si="3"/>
@@ -38115,7 +38515,7 @@
       </c>
       <c r="G25" s="2">
         <f t="shared" si="2"/>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H25" s="6">
         <f>I25+개인기록Sheet!C59</f>
@@ -38229,11 +38629,11 @@
       </c>
       <c r="G26" s="2">
         <f t="shared" si="2"/>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H26" s="6">
         <f>I26+개인기록Sheet!C60</f>
-        <v>4.5999999999999996</v>
+        <v>4.8</v>
       </c>
       <c r="I26" s="6">
         <f t="shared" si="3"/>
@@ -38907,7 +39307,7 @@
       </c>
       <c r="G32" s="2">
         <f t="shared" si="2"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H32" s="6">
         <f>I32+개인기록Sheet!C79</f>
@@ -39027,7 +39427,7 @@
       </c>
       <c r="H33" s="6">
         <f>I33+개인기록Sheet!C83</f>
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="I33" s="6">
         <f t="shared" si="6"/>
@@ -39361,11 +39761,11 @@
       </c>
       <c r="G36" s="2">
         <f t="shared" si="2"/>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H36" s="6">
         <f>I36+개인기록Sheet!C102</f>
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="I36" s="6">
         <f t="shared" si="6"/>
@@ -39479,7 +39879,7 @@
       </c>
       <c r="H37" s="6">
         <f>I37+개인기록Sheet!C104</f>
-        <v>8</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="I37" s="6">
         <f t="shared" si="6"/>

</xml_diff>